<commit_message>
fix: re-resolve web upstream via Docker DNS so the proxy survives container restarts (V2.6)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R4a6688ec04ab441a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rfcf6156e888741bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R23be06e9d85640b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R6c0d05c3c4b042ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R682b931bbcc348e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rf46ab81e404f4648"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -659,23 +659,43 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="15" t="str">
+      <x:c r="A14" s="11" t="str">
         <x:v>V2.5</x:v>
       </x:c>
-      <x:c r="B14" s="16" t="n">
+      <x:c r="B14" s="12" t="n">
         <x:v>46282</x:v>
       </x:c>
-      <x:c r="C14" s="17" t="str">
+      <x:c r="C14" s="13" t="str">
         <x:v>小型修改</x:v>
       </x:c>
-      <x:c r="D14" s="17" t="str">
+      <x:c r="D14" s="13" t="str">
         <x:v>建立版本管理规则：新增 VERSION 版本号文件、本变更说明表、AGENTS.md 版本与变更记录规则；为历史版本补打 Git 标签</x:v>
       </x:c>
-      <x:c r="E14" s="17" t="str">
+      <x:c r="E14" s="13" t="str">
         <x:v>本次提交, 标签 v2.5</x:v>
       </x:c>
-      <x:c r="F14" s="18" t="str">
+      <x:c r="F14" s="13" t="str">
         <x:v>规则文档与变更表落地；GitHub 标签与提交同步完成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="33" t="str">
+        <x:v>V2.6</x:v>
+      </x:c>
+      <x:c r="B15" s="35" t="n">
+        <x:v>46282</x:v>
+      </x:c>
+      <x:c r="C15" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D15" s="34" t="str">
+        <x:v>修复代理缓存旧 IP 导致界面 502：nginx 改用 Docker 内嵌 DNS（127.0.0.11, valid=10s）重新解析后端，容器重建后不再断链</x:v>
+      </x:c>
+      <x:c r="E15" s="34" t="str">
+        <x:v>本次提交, 标签 v2.6</x:v>
+      </x:c>
+      <x:c r="F15" s="34" t="str">
+        <x:v>重启 web 容器后代理仍返回 200；局域网登录页与健康检查通过</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -867,17 +887,31 @@
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="33" t="str">
+      <x:c r="A15" s="29" t="str">
         <x:v>V2.5</x:v>
       </x:c>
-      <x:c r="B15" s="34" t="str">
+      <x:c r="B15" s="30" t="str">
         <x:v>（本次提交）</x:v>
       </x:c>
-      <x:c r="C15" s="35" t="n">
+      <x:c r="C15" s="31" t="n">
         <x:v>46282</x:v>
       </x:c>
-      <x:c r="D15" s="36" t="str">
+      <x:c r="D15" s="30" t="str">
         <x:v>docs: 建立版本号与变更说明规则</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="33" t="str">
+        <x:v>V2.6</x:v>
+      </x:c>
+      <x:c r="B16" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C16" s="35" t="n">
+        <x:v>46282</x:v>
+      </x:c>
+      <x:c r="D16" s="34" t="str">
+        <x:v>fix: 代理改用 Docker 内嵌 DNS 重新解析后端，修复容器重建后 502</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
chore: record role test accounts in change log (V2.6)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R6c0d05c3c4b042ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R682b931bbcc348e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rf46ab81e404f4648"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R84fe758cd1714bd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rf0f61ceae26a4ffd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R6be9785efc3842d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -679,23 +679,43 @@
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="33" t="str">
+      <x:c r="A15" s="29" t="str">
         <x:v>V2.6</x:v>
       </x:c>
-      <x:c r="B15" s="35" t="n">
+      <x:c r="B15" s="31" t="n">
         <x:v>46282</x:v>
       </x:c>
-      <x:c r="C15" s="34" t="str">
+      <x:c r="C15" s="30" t="str">
         <x:v>小型修改</x:v>
       </x:c>
-      <x:c r="D15" s="34" t="str">
+      <x:c r="D15" s="30" t="str">
         <x:v>修复代理缓存旧 IP 导致界面 502：nginx 改用 Docker 内嵌 DNS（127.0.0.11, valid=10s）重新解析后端，容器重建后不再断链</x:v>
       </x:c>
-      <x:c r="E15" s="34" t="str">
+      <x:c r="E15" s="30" t="str">
         <x:v>本次提交, 标签 v2.6</x:v>
       </x:c>
-      <x:c r="F15" s="34" t="str">
+      <x:c r="F15" s="30" t="str">
         <x:v>重启 web 容器后代理仍返回 200；局域网登录页与健康检查通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="33" t="str">
+        <x:v>V2.6</x:v>
+      </x:c>
+      <x:c r="B16" s="35" t="n">
+        <x:v>46282</x:v>
+      </x:c>
+      <x:c r="C16" s="34" t="str">
+        <x:v>数据变更</x:v>
+      </x:c>
+      <x:c r="D16" s="34" t="str">
+        <x:v>部署库新增三种权限的测试账号：编辑者 editor、阅读者 reader（按 AUTH-02 首登强制改密）；管理员沿用 qadmin</x:v>
+      </x:c>
+      <x:c r="E16" s="34" t="str">
+        <x:v>无（数据库操作，未改代码）</x:v>
+      </x:c>
+      <x:c r="F16" s="34" t="str">
+        <x:v>四种账号密码验证通过（qadmin/reader/editor 可直接登录）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
ops: add wizard to fix the portal LAN address on wired Ethernet (V2.6)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R84fe758cd1714bd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rf0f61ceae26a4ffd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R6be9785efc3842d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R3853e8981a854cf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Re140ada9adfb45a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R1eb26e792ce2419e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -699,23 +699,43 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="33" t="str">
+      <x:c r="A16" s="29" t="str">
         <x:v>V2.6</x:v>
       </x:c>
-      <x:c r="B16" s="35" t="n">
+      <x:c r="B16" s="31" t="n">
         <x:v>46282</x:v>
       </x:c>
-      <x:c r="C16" s="34" t="str">
+      <x:c r="C16" s="30" t="str">
         <x:v>数据变更</x:v>
       </x:c>
-      <x:c r="D16" s="34" t="str">
+      <x:c r="D16" s="30" t="str">
         <x:v>部署库新增三种权限的测试账号：编辑者 editor、阅读者 reader（按 AUTH-02 首登强制改密）；管理员沿用 qadmin</x:v>
       </x:c>
-      <x:c r="E16" s="34" t="str">
+      <x:c r="E16" s="30" t="str">
         <x:v>无（数据库操作，未改代码）</x:v>
       </x:c>
-      <x:c r="F16" s="34" t="str">
+      <x:c r="F16" s="30" t="str">
         <x:v>四种账号密码验证通过（qadmin/reader/editor 可直接登录）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="33" t="str">
+        <x:v>V2.6</x:v>
+      </x:c>
+      <x:c r="B17" s="35" t="n">
+        <x:v>46282</x:v>
+      </x:c>
+      <x:c r="C17" s="34" t="str">
+        <x:v>环境变更</x:v>
+      </x:c>
+      <x:c r="D17" s="34" t="str">
+        <x:v>新增 scripts/configure-wired-lan-ip.sh 向导：把门户局域网地址固定在有线以太网 en0（192.168.60.152/22，网关 192.168.60.1），避免 DHCP 重新分配导致地址失效；WiFi 不受影响</x:v>
+      </x:c>
+      <x:c r="E17" s="34" t="str">
+        <x:v>本次提交</x:v>
+      </x:c>
+      <x:c r="F17" s="34" t="str">
+        <x:v>向导含静态地址设置、服务可达性验证与回滚说明（需管理员密码执行）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix: allow editors to maintain the onboarding route (V2.7)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R3853e8981a854cf7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Re140ada9adfb45a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R1eb26e792ce2419e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rcf38cd79183943cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rc20bbbf6d1f54d48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rae5d30e9dc9845e2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -719,23 +719,43 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="33" t="str">
+      <x:c r="A17" s="29" t="str">
         <x:v>V2.6</x:v>
       </x:c>
-      <x:c r="B17" s="35" t="n">
+      <x:c r="B17" s="31" t="n">
         <x:v>46282</x:v>
       </x:c>
-      <x:c r="C17" s="34" t="str">
+      <x:c r="C17" s="30" t="str">
         <x:v>环境变更</x:v>
       </x:c>
-      <x:c r="D17" s="34" t="str">
+      <x:c r="D17" s="30" t="str">
         <x:v>新增 scripts/configure-wired-lan-ip.sh 向导：把门户局域网地址固定在有线以太网 en0（192.168.60.152/22，网关 192.168.60.1），避免 DHCP 重新分配导致地址失效；WiFi 不受影响</x:v>
       </x:c>
-      <x:c r="E17" s="34" t="str">
+      <x:c r="E17" s="30" t="str">
         <x:v>本次提交</x:v>
       </x:c>
-      <x:c r="F17" s="34" t="str">
+      <x:c r="F17" s="30" t="str">
         <x:v>向导含静态地址设置、服务可达性验证与回滚说明（需管理员密码执行）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="33" t="str">
+        <x:v>V2.7</x:v>
+      </x:c>
+      <x:c r="B18" s="35" t="n">
+        <x:v>46282</x:v>
+      </x:c>
+      <x:c r="C18" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D18" s="34" t="str">
+        <x:v>修复权限缺陷：新人路线管理（新人专区）原先仅管理员可进入且模块仅允许管理员，与需求「编辑者可维护学习路线」不符；现开放给编辑者，阅读者仍被拒绝</x:v>
+      </x:c>
+      <x:c r="E18" s="34" t="str">
+        <x:v>本次提交, 标签 v2.7</x:v>
+      </x:c>
+      <x:c r="F18" s="34" t="str">
+        <x:v>模块测试与 e2e 更新并通过；线上实例以编辑者身份实际更新阶段说明成功（阅读者仍被拒绝）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -941,17 +961,31 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="33" t="str">
+      <x:c r="A16" s="29" t="str">
         <x:v>V2.6</x:v>
       </x:c>
-      <x:c r="B16" s="34" t="str">
+      <x:c r="B16" s="30" t="str">
         <x:v>（本次提交）</x:v>
       </x:c>
-      <x:c r="C16" s="35" t="n">
+      <x:c r="C16" s="31" t="n">
         <x:v>46282</x:v>
       </x:c>
-      <x:c r="D16" s="34" t="str">
+      <x:c r="D16" s="30" t="str">
         <x:v>fix: 代理改用 Docker 内嵌 DNS 重新解析后端，修复容器重建后 502</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="33" t="str">
+        <x:v>V2.7</x:v>
+      </x:c>
+      <x:c r="B17" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C17" s="35" t="n">
+        <x:v>46282</x:v>
+      </x:c>
+      <x:c r="D17" s="34" t="str">
+        <x:v>fix: 新人专区（学习路线）维护权限按需求开放给编辑者</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix: add editor management entries and open column management to editors (V2.8)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rcf38cd79183943cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rc20bbbf6d1f54d48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rae5d30e9dc9845e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R6f3a2d5d9982433b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R36c5b0763cf04940"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R71a53b83d59d4feb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -739,23 +739,43 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="33" t="str">
+      <x:c r="A18" s="29" t="str">
         <x:v>V2.7</x:v>
       </x:c>
-      <x:c r="B18" s="35" t="n">
+      <x:c r="B18" s="31" t="n">
         <x:v>46282</x:v>
       </x:c>
-      <x:c r="C18" s="34" t="str">
+      <x:c r="C18" s="30" t="str">
         <x:v>小型修改</x:v>
       </x:c>
-      <x:c r="D18" s="34" t="str">
+      <x:c r="D18" s="30" t="str">
         <x:v>修复权限缺陷：新人路线管理（新人专区）原先仅管理员可进入且模块仅允许管理员，与需求「编辑者可维护学习路线」不符；现开放给编辑者，阅读者仍被拒绝</x:v>
       </x:c>
-      <x:c r="E18" s="34" t="str">
+      <x:c r="E18" s="30" t="str">
         <x:v>本次提交, 标签 v2.7</x:v>
       </x:c>
-      <x:c r="F18" s="34" t="str">
+      <x:c r="F18" s="30" t="str">
         <x:v>模块测试与 e2e 更新并通过；线上实例以编辑者身份实际更新阶段说明成功（阅读者仍被拒绝）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="33" t="str">
+        <x:v>V2.8</x:v>
+      </x:c>
+      <x:c r="B19" s="35" t="n">
+        <x:v>46282</x:v>
+      </x:c>
+      <x:c r="C19" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D19" s="34" t="str">
+        <x:v>编辑者「管理」落地页补齐「新人路线管理」「栏目与主题管理」入口（此前只有权限无入口）；栏目与主题管理按用户要求开放给编辑者（阅读者仍拒绝），并同步更新需求文档角色能力表、IA-07 与 CONTEXT.md 职责描述</x:v>
+      </x:c>
+      <x:c r="E19" s="34" t="str">
+        <x:v>本次提交, 标签 v2.8</x:v>
+      </x:c>
+      <x:c r="F19" s="34" t="str">
+        <x:v>全量测试 281 用例通过；线上实例以编辑者身份验证：落地页入口可见、新人路线管理可访问、栏目改名成功（已还原）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -975,17 +995,31 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="33" t="str">
+      <x:c r="A17" s="29" t="str">
         <x:v>V2.7</x:v>
       </x:c>
-      <x:c r="B17" s="34" t="str">
+      <x:c r="B17" s="30" t="str">
         <x:v>（本次提交）</x:v>
       </x:c>
-      <x:c r="C17" s="35" t="n">
+      <x:c r="C17" s="31" t="n">
         <x:v>46282</x:v>
       </x:c>
-      <x:c r="D17" s="34" t="str">
+      <x:c r="D17" s="30" t="str">
         <x:v>fix: 新人专区（学习路线）维护权限按需求开放给编辑者</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="33" t="str">
+        <x:v>V2.8</x:v>
+      </x:c>
+      <x:c r="B18" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C18" s="35" t="n">
+        <x:v>46282</x:v>
+      </x:c>
+      <x:c r="D18" s="34" t="str">
+        <x:v>fix: 编辑者管理入口补齐 + 栏目与主题管理权限开放给编辑者</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix: complete the article maintenance flow for editors (V2.9)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R6f3a2d5d9982433b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R36c5b0763cf04940"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R71a53b83d59d4feb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rba523220e4214f42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R61a6a413498c4703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rd341f7d4ea6f4230"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -759,23 +759,43 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="33" t="str">
+      <x:c r="A19" s="29" t="str">
         <x:v>V2.8</x:v>
       </x:c>
-      <x:c r="B19" s="35" t="n">
+      <x:c r="B19" s="31" t="n">
         <x:v>46282</x:v>
       </x:c>
-      <x:c r="C19" s="34" t="str">
+      <x:c r="C19" s="30" t="str">
         <x:v>小型修改</x:v>
       </x:c>
-      <x:c r="D19" s="34" t="str">
+      <x:c r="D19" s="30" t="str">
         <x:v>编辑者「管理」落地页补齐「新人路线管理」「栏目与主题管理」入口（此前只有权限无入口）；栏目与主题管理按用户要求开放给编辑者（阅读者仍拒绝），并同步更新需求文档角色能力表、IA-07 与 CONTEXT.md 职责描述</x:v>
       </x:c>
-      <x:c r="E19" s="34" t="str">
+      <x:c r="E19" s="30" t="str">
         <x:v>本次提交, 标签 v2.8</x:v>
       </x:c>
-      <x:c r="F19" s="34" t="str">
+      <x:c r="F19" s="30" t="str">
         <x:v>全量测试 281 用例通过；线上实例以编辑者身份验证：落地页入口可见、新人路线管理可访问、栏目改名成功（已还原）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="33" t="str">
+        <x:v>V2.9</x:v>
+      </x:c>
+      <x:c r="B20" s="35" t="n">
+        <x:v>46282</x:v>
+      </x:c>
+      <x:c r="C20" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D20" s="34" t="str">
+        <x:v>补齐文章维护闭环：新增「文章管理」列表页（按状态筛选）与管理入口；「新建文章」页接上创建草稿动作（此前点保存无任何反应）；编辑器新增「知识别名」字段（IA-06）；内容负责人由手填 UUID 改为账号下拉；保存后显示提示条</x:v>
+      </x:c>
+      <x:c r="E20" s="34" t="str">
+        <x:v>本次提交, 标签 v2.9</x:v>
+      </x:c>
+      <x:c r="F20" s="34" t="str">
+        <x:v>全量测试 283 用例、e2e 新增文章维护用例通过；线上以编辑者身份实测：进入文章管理→新建→填写含别名→保存草稿→出现在草稿列表</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1009,17 +1029,31 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="33" t="str">
+      <x:c r="A18" s="29" t="str">
         <x:v>V2.8</x:v>
       </x:c>
-      <x:c r="B18" s="34" t="str">
+      <x:c r="B18" s="30" t="str">
         <x:v>（本次提交）</x:v>
       </x:c>
-      <x:c r="C18" s="35" t="n">
+      <x:c r="C18" s="31" t="n">
         <x:v>46282</x:v>
       </x:c>
-      <x:c r="D18" s="34" t="str">
+      <x:c r="D18" s="30" t="str">
         <x:v>fix: 编辑者管理入口补齐 + 栏目与主题管理权限开放给编辑者</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="33" t="str">
+        <x:v>V2.9</x:v>
+      </x:c>
+      <x:c r="B19" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C19" s="35" t="n">
+        <x:v>46282</x:v>
+      </x:c>
+      <x:c r="D19" s="34" t="str">
+        <x:v>fix: 文章管理列表与入口、新建文章保存动作、知识别名与负责人下拉</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: manage onboarding as ordered articles (V3.0)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rba523220e4214f42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R61a6a413498c4703"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rd341f7d4ea6f4230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Re41c3c7cfb2943fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rf4fe6d7060574d73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R80ea79a8b2f04539"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -798,6 +798,26 @@
         <x:v>全量测试 283 用例、e2e 新增文章维护用例通过；线上以编辑者身份实测：进入文章管理→新建→填写含别名→保存草稿→出现在草稿列表</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>V3.0</x:v>
+      </x:c>
+      <x:c r="B21" t="n">
+        <x:v>46283</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>Superpower 需求</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>新人路线改为一篇文章对应一步的可编辑列表，支持搜索添加、新建、编辑、排序和移出；原阶段内容与链接无损迁移，数量不再固定为六步；文章创建与路线加入同一事务，草稿与发布保留上一版。</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>本次提交，标签 v3.0</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>Vitest 迁移/路线/版本回归通过；Playwright 新人路线与文章维护 10 场景通过；typecheck、lint、build 通过；PostgreSQL 容器验证通过。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1056,6 +1076,20 @@
         <x:v>fix: 文章管理列表与入口、新建文章保存动作、知识别名与负责人下拉</x:v>
       </x:c>
     </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>V3.0</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C20" t="n">
+        <x:v>46283</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>feat: 新人路线改为可编辑文章列表，迁移旧阶段并保证原子创建与版本快照</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix: publish drafts directly from the article and route lists (V3.1)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Re41c3c7cfb2943fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rf4fe6d7060574d73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R80ea79a8b2f04539"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R9f6fcc59e4734a6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R8d84233da71841d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R469417821f674896"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -799,23 +799,43 @@
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" t="str">
+      <x:c r="A21" s="26" t="str">
         <x:v>V3.0</x:v>
       </x:c>
-      <x:c r="B21" t="n">
+      <x:c r="B21" s="27" t="n">
         <x:v>46283</x:v>
       </x:c>
-      <x:c r="C21" t="str">
+      <x:c r="C21" s="27" t="str">
         <x:v>Superpower 需求</x:v>
       </x:c>
-      <x:c r="D21" t="str">
+      <x:c r="D21" s="27" t="str">
         <x:v>新人路线改为一篇文章对应一步的可编辑列表，支持搜索添加、新建、编辑、排序和移出；原阶段内容与链接无损迁移，数量不再固定为六步；文章创建与路线加入同一事务，草稿与发布保留上一版。</x:v>
       </x:c>
-      <x:c r="E21" t="str">
+      <x:c r="E21" s="27" t="str">
         <x:v>本次提交，标签 v3.0</x:v>
       </x:c>
-      <x:c r="F21" t="str">
+      <x:c r="F21" s="28" t="str">
         <x:v>Vitest 迁移/路线/版本回归通过；Playwright 新人路线与文章维护 10 场景通过；typecheck、lint、build 通过；PostgreSQL 容器验证通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="33" t="str">
+        <x:v>V3.1</x:v>
+      </x:c>
+      <x:c r="B22" s="35" t="n">
+        <x:v>46283</x:v>
+      </x:c>
+      <x:c r="C22" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D22" s="34" t="str">
+        <x:v>草稿箱补齐发布入口：文章管理列表的草稿行与新人路线列表的草稿行新增「发布」按钮，不必先打开编辑器即可发布（此前发布按钮只存在于编辑器属性面板，草稿在列表里无法发布）；发布失败时按缺项给出提示，案例文章提示先到编辑器确认脱敏；发布成功后提示并刷新阅读侧</x:v>
+      </x:c>
+      <x:c r="E22" s="34" t="str">
+        <x:v>本次提交，标签 v3.1</x:v>
+      </x:c>
+      <x:c r="F22" s="36" t="str">
+        <x:v>新增 4 条 e2e 回归（列表发布成功并阅读侧可见、缺必填项报错且状态不变、新人路线列表发布、读者无权进入）；全量 281 单元用例与新增 e2e 通过；以编辑者身份在部署实例实测草稿箱直接发布成功</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1077,17 +1097,31 @@
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" t="str">
+      <x:c r="A20" s="26" t="str">
         <x:v>V3.0</x:v>
       </x:c>
-      <x:c r="B20" t="str">
+      <x:c r="B20" s="27" t="str">
         <x:v>（本次提交）</x:v>
       </x:c>
-      <x:c r="C20" t="n">
+      <x:c r="C20" s="27" t="n">
         <x:v>46283</x:v>
       </x:c>
-      <x:c r="D20" t="str">
+      <x:c r="D20" s="28" t="str">
         <x:v>feat: 新人路线改为可编辑文章列表，迁移旧阶段并保证原子创建与版本快照</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="33" t="str">
+        <x:v>V3.1</x:v>
+      </x:c>
+      <x:c r="B21" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C21" s="35" t="n">
+        <x:v>46283</x:v>
+      </x:c>
+      <x:c r="D21" s="36" t="str">
+        <x:v>fix: 列表页补齐草稿发布入口（文章管理与新人路线）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: render whole article bodies inline on topic pages (V3.2)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R9f6fcc59e4734a6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R8d84233da71841d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R469417821f674896"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rfcd9dcf375a64b6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R867170557d794c59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rc13b10fc5bd24f42"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -819,23 +819,43 @@
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="33" t="str">
+      <x:c r="A22" s="29" t="str">
         <x:v>V3.1</x:v>
       </x:c>
-      <x:c r="B22" s="35" t="n">
+      <x:c r="B22" s="31" t="n">
         <x:v>46283</x:v>
       </x:c>
-      <x:c r="C22" s="34" t="str">
+      <x:c r="C22" s="30" t="str">
         <x:v>小型修改</x:v>
       </x:c>
-      <x:c r="D22" s="34" t="str">
+      <x:c r="D22" s="30" t="str">
         <x:v>草稿箱补齐发布入口：文章管理列表的草稿行与新人路线列表的草稿行新增「发布」按钮，不必先打开编辑器即可发布（此前发布按钮只存在于编辑器属性面板，草稿在列表里无法发布）；发布失败时按缺项给出提示，案例文章提示先到编辑器确认脱敏；发布成功后提示并刷新阅读侧</x:v>
       </x:c>
-      <x:c r="E22" s="34" t="str">
+      <x:c r="E22" s="30" t="str">
         <x:v>本次提交，标签 v3.1</x:v>
       </x:c>
-      <x:c r="F22" s="36" t="str">
+      <x:c r="F22" s="30" t="str">
         <x:v>新增 4 条 e2e 回归（列表发布成功并阅读侧可见、缺必填项报错且状态不变、新人路线列表发布、读者无权进入）；全量 281 单元用例与新增 e2e 通过；以编辑者身份在部署实例实测草稿箱直接发布成功</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="33" t="str">
+        <x:v>V3.2</x:v>
+      </x:c>
+      <x:c r="B23" s="35" t="n">
+        <x:v>46283</x:v>
+      </x:c>
+      <x:c r="C23" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D23" s="34" t="str">
+        <x:v>主题页改为整篇可读：品质知识 / 散热知识的主题页内联渲染每篇已发布文章的完整正文（此前只显示标题与摘要，需要另点一次才能阅读）；文章标题改为可见链接并新增「打开阅读页（目录 / 收藏 / 反馈）」入口；正文渲染抽成阅读页与主题页共用的 ArticleBody 组件；同时修复正文图片缺少宽度约束把整页撑出横向滚动的问题（阅读页与主题页一并生效）；草稿与已归档文章仍不进入阅读侧</x:v>
+      </x:c>
+      <x:c r="E23" s="34" t="str">
+        <x:v>本次提交，标签 v3.2</x:v>
+      </x:c>
+      <x:c r="F23" s="34" t="str">
+        <x:v>新增模块用例（主题页正文列表含正文、排除草稿与归档）与 e2e（主题页内联正文可见、窄屏无横向滚动、仍可进入阅读页）；全量 282 单元用例、9 个 PostgreSQL 容器用例、84 条 e2e 通过；线上以管理员身份实测主题页显示整篇正文</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1111,17 +1131,31 @@
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="33" t="str">
+      <x:c r="A21" s="29" t="str">
         <x:v>V3.1</x:v>
       </x:c>
-      <x:c r="B21" s="34" t="str">
+      <x:c r="B21" s="30" t="str">
         <x:v>（本次提交）</x:v>
       </x:c>
-      <x:c r="C21" s="35" t="n">
+      <x:c r="C21" s="31" t="n">
         <x:v>46283</x:v>
       </x:c>
-      <x:c r="D21" s="36" t="str">
+      <x:c r="D21" s="30" t="str">
         <x:v>fix: 列表页补齐草稿发布入口（文章管理与新人路线）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="33" t="str">
+        <x:v>V3.2</x:v>
+      </x:c>
+      <x:c r="B22" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C22" s="35" t="n">
+        <x:v>46283</x:v>
+      </x:c>
+      <x:c r="D22" s="34" t="str">
+        <x:v>feat: 主题页内联渲染整篇正文（共用 ArticleBody 组件）并约束正文图片宽度</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
refactor: trim the topic page down to owner/update line plus body (V3.3)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rfcd9dcf375a64b6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R867170557d794c59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rc13b10fc5bd24f42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R7d6990a7bf544ae6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rc00d4b6f369f4c7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rf48e4978e3244147"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -839,23 +839,43 @@
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="33" t="str">
+      <x:c r="A23" s="29" t="str">
         <x:v>V3.2</x:v>
       </x:c>
-      <x:c r="B23" s="35" t="n">
+      <x:c r="B23" s="31" t="n">
         <x:v>46283</x:v>
       </x:c>
-      <x:c r="C23" s="34" t="str">
+      <x:c r="C23" s="30" t="str">
         <x:v>小型修改</x:v>
       </x:c>
-      <x:c r="D23" s="34" t="str">
+      <x:c r="D23" s="30" t="str">
         <x:v>主题页改为整篇可读：品质知识 / 散热知识的主题页内联渲染每篇已发布文章的完整正文（此前只显示标题与摘要，需要另点一次才能阅读）；文章标题改为可见链接并新增「打开阅读页（目录 / 收藏 / 反馈）」入口；正文渲染抽成阅读页与主题页共用的 ArticleBody 组件；同时修复正文图片缺少宽度约束把整页撑出横向滚动的问题（阅读页与主题页一并生效）；草稿与已归档文章仍不进入阅读侧</x:v>
       </x:c>
-      <x:c r="E23" s="34" t="str">
+      <x:c r="E23" s="30" t="str">
         <x:v>本次提交，标签 v3.2</x:v>
       </x:c>
-      <x:c r="F23" s="34" t="str">
+      <x:c r="F23" s="30" t="str">
         <x:v>新增模块用例（主题页正文列表含正文、排除草稿与归档）与 e2e（主题页内联正文可见、窄屏无横向滚动、仍可进入阅读页）；全量 282 单元用例、9 个 PostgreSQL 容器用例、84 条 e2e 通过；线上以管理员身份实测主题页显示整篇正文</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="33" t="str">
+        <x:v>V3.3</x:v>
+      </x:c>
+      <x:c r="B24" s="35" t="n">
+        <x:v>46283</x:v>
+      </x:c>
+      <x:c r="C24" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D24" s="34" t="str">
+        <x:v>主题页信息层级精简：正文区上方重复的「品质知识」栏目名、Mean / σ 之类主题名、文章标题与摘要全部去掉，主题页只保留「负责人 · 更新时间 · 打开阅读页（目录 / 收藏 / 反馈）」一行加整篇 Markdown 正文（栏目与主题已由顶部导航和左侧分类树表达）；为无障碍保留屏幕阅读器可见的栏目名 / 主题名 / 文章标题结构，视觉上不占位</x:v>
+      </x:c>
+      <x:c r="E24" s="34" t="str">
+        <x:v>本次提交，标签 v3.3</x:v>
+      </x:c>
+      <x:c r="F24" s="34" t="str">
+        <x:v>e2e 更新为断言可见证据（顶部导航 aria-current、分类树选中态、正文文本、摘要不再出现）；全量 282 单元用例、9 个 PostgreSQL 容器用例、84 条 e2e 通过；线上以管理员身份实测主题页正文区只剩负责人/更新时间一行加整篇正文，1280px 与 390px 均无横向滚动</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1145,17 +1165,31 @@
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="33" t="str">
+      <x:c r="A22" s="29" t="str">
         <x:v>V3.2</x:v>
       </x:c>
-      <x:c r="B22" s="34" t="str">
+      <x:c r="B22" s="30" t="str">
         <x:v>（本次提交）</x:v>
       </x:c>
-      <x:c r="C22" s="35" t="n">
+      <x:c r="C22" s="31" t="n">
         <x:v>46283</x:v>
       </x:c>
-      <x:c r="D22" s="34" t="str">
+      <x:c r="D22" s="30" t="str">
         <x:v>feat: 主题页内联渲染整篇正文（共用 ArticleBody 组件）并约束正文图片宽度</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="33" t="str">
+        <x:v>V3.3</x:v>
+      </x:c>
+      <x:c r="B23" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C23" s="35" t="n">
+        <x:v>46283</x:v>
+      </x:c>
+      <x:c r="D23" s="34" t="str">
+        <x:v>refactor: 精简主题页信息层级，正文区只留负责人/更新时间与正文</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: archive articles from the management list (V3.4)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R7d6990a7bf544ae6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rc00d4b6f369f4c7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rf48e4978e3244147"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R7645c9945166444c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R5044ebd456224ac5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rcae6f8a7248e4734"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -859,23 +859,43 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="33" t="str">
+      <x:c r="A24" s="29" t="str">
         <x:v>V3.3</x:v>
       </x:c>
-      <x:c r="B24" s="35" t="n">
+      <x:c r="B24" s="31" t="n">
         <x:v>46283</x:v>
       </x:c>
-      <x:c r="C24" s="34" t="str">
+      <x:c r="C24" s="30" t="str">
         <x:v>小型修改</x:v>
       </x:c>
-      <x:c r="D24" s="34" t="str">
+      <x:c r="D24" s="30" t="str">
         <x:v>主题页信息层级精简：正文区上方重复的「品质知识」栏目名、Mean / σ 之类主题名、文章标题与摘要全部去掉，主题页只保留「负责人 · 更新时间 · 打开阅读页（目录 / 收藏 / 反馈）」一行加整篇 Markdown 正文（栏目与主题已由顶部导航和左侧分类树表达）；为无障碍保留屏幕阅读器可见的栏目名 / 主题名 / 文章标题结构，视觉上不占位</x:v>
       </x:c>
-      <x:c r="E24" s="34" t="str">
+      <x:c r="E24" s="30" t="str">
         <x:v>本次提交，标签 v3.3</x:v>
       </x:c>
-      <x:c r="F24" s="34" t="str">
+      <x:c r="F24" s="30" t="str">
         <x:v>e2e 更新为断言可见证据（顶部导航 aria-current、分类树选中态、正文文本、摘要不再出现）；全量 282 单元用例、9 个 PostgreSQL 容器用例、84 条 e2e 通过；线上以管理员身份实测主题页正文区只剩负责人/更新时间一行加整篇正文，1280px 与 390px 均无横向滚动</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="33" t="str">
+        <x:v>V3.4</x:v>
+      </x:c>
+      <x:c r="B25" s="35" t="n">
+        <x:v>46285</x:v>
+      </x:c>
+      <x:c r="C25" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D25" s="34" t="str">
+        <x:v>文章管理列表补齐归档入口：每行直接填写归档原因即可归档（此前归档按钮只藏在「版本历史」页，文章管理列表里找不到，测试文章无法撤下）；归档后文章立刻从阅读侧（主题页、首页最近更新）和列表撤下并进入回收站，符合 DEL-01/DEL-02（日常删除用归档，回收站保留 30 天后才允许管理员永久清理）；管理员可在文章管理页直达回收站，已归档内容在「已归档」筛选下可查</x:v>
+      </x:c>
+      <x:c r="E25" s="34" t="str">
+        <x:v>本次提交，标签 v3.4</x:v>
+      </x:c>
+      <x:c r="F25" s="34" t="str">
+        <x:v>新增 e2e：编辑者在列表页归档测试文章 → 阅读侧不再展示、旧链接给归档说明、回收站可见且永久删除按钮禁用、管理员恢复后可回到草稿箱；全量 282 单元用例、9 个 PostgreSQL 容器用例、85 条 e2e 通过；窄屏无横向滚动</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1179,17 +1199,31 @@
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="33" t="str">
+      <x:c r="A23" s="29" t="str">
         <x:v>V3.3</x:v>
       </x:c>
-      <x:c r="B23" s="34" t="str">
+      <x:c r="B23" s="30" t="str">
         <x:v>（本次提交）</x:v>
       </x:c>
-      <x:c r="C23" s="35" t="n">
+      <x:c r="C23" s="31" t="n">
         <x:v>46283</x:v>
       </x:c>
-      <x:c r="D23" s="34" t="str">
+      <x:c r="D23" s="30" t="str">
         <x:v>refactor: 精简主题页信息层级，正文区只留负责人/更新时间与正文</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="33" t="str">
+        <x:v>V3.4</x:v>
+      </x:c>
+      <x:c r="B24" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C24" s="35" t="n">
+        <x:v>46285</x:v>
+      </x:c>
+      <x:c r="D24" s="34" t="str">
+        <x:v>feat: 文章管理列表补齐归档入口（含归档原因与回收站入口）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: allow admins to purge never-published drafts immediately (V3.5)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R7645c9945166444c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R5044ebd456224ac5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rcae6f8a7248e4734"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R0744ae9eeb534ce3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rc21168e7e9cd4c9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R7488e54e31b84a28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -879,23 +879,43 @@
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="33" t="str">
+      <x:c r="A25" s="29" t="str">
         <x:v>V3.4</x:v>
       </x:c>
-      <x:c r="B25" s="35" t="n">
+      <x:c r="B25" s="31" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="C25" s="34" t="str">
-        <x:v>小型修改</x:v>
-      </x:c>
-      <x:c r="D25" s="34" t="str">
+      <x:c r="C25" s="30" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D25" s="30" t="str">
         <x:v>文章管理列表补齐归档入口：每行直接填写归档原因即可归档（此前归档按钮只藏在「版本历史」页，文章管理列表里找不到，测试文章无法撤下）；归档后文章立刻从阅读侧（主题页、首页最近更新）和列表撤下并进入回收站，符合 DEL-01/DEL-02（日常删除用归档，回收站保留 30 天后才允许管理员永久清理）；管理员可在文章管理页直达回收站，已归档内容在「已归档」筛选下可查</x:v>
       </x:c>
-      <x:c r="E25" s="34" t="str">
+      <x:c r="E25" s="30" t="str">
         <x:v>本次提交，标签 v3.4</x:v>
       </x:c>
-      <x:c r="F25" s="34" t="str">
+      <x:c r="F25" s="30" t="str">
         <x:v>新增 e2e：编辑者在列表页归档测试文章 → 阅读侧不再展示、旧链接给归档说明、回收站可见且永久删除按钮禁用、管理员恢复后可回到草稿箱；全量 282 单元用例、9 个 PostgreSQL 容器用例、85 条 e2e 通过；窄屏无横向滚动</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="33" t="str">
+        <x:v>V3.5</x:v>
+      </x:c>
+      <x:c r="B26" s="35" t="n">
+        <x:v>46285</x:v>
+      </x:c>
+      <x:c r="C26" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D26" s="34" t="str">
+        <x:v>按用户确认放宽永久清理规则：从未发布过的草稿可由管理员在回收站立即永久删除，删除必须填写原因并写入审计（规则标记 never-published-draft）；已发布过的内容仍保留 30 天才能清理，避免读者侧内容被误删。回收站列表对可立即删除的条目显示原因提示与删除原因输入框，删除失败改为错误提示；同步更新需求文档 DEL-02、验收准则与 CONTEXT 的措辞</x:v>
+      </x:c>
+      <x:c r="E26" s="34" t="str">
+        <x:v>本次提交，标签 v3.5</x:v>
+      </x:c>
+      <x:c r="F26" s="34" t="str">
+        <x:v>模块用例覆盖：未发布草稿可立即删除且写审计（含 rule 字段）、空白原因被拒、已发布内容仍报「保留 30 天」；e2e 覆盖编辑者归档→管理员带原因永久删除→列表与阅读侧彻底消失；全量 283 单元用例、9 个 PostgreSQL 容器用例、86 条 e2e 通过；线上实测完整走通一次（含审计留痕）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1213,17 +1233,31 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="33" t="str">
+      <x:c r="A24" s="29" t="str">
         <x:v>V3.4</x:v>
       </x:c>
-      <x:c r="B24" s="34" t="str">
+      <x:c r="B24" s="30" t="str">
         <x:v>（本次提交）</x:v>
       </x:c>
-      <x:c r="C24" s="35" t="n">
+      <x:c r="C24" s="31" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="D24" s="34" t="str">
+      <x:c r="D24" s="30" t="str">
         <x:v>feat: 文章管理列表补齐归档入口（含归档原因与回收站入口）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="33" t="str">
+        <x:v>V3.5</x:v>
+      </x:c>
+      <x:c r="B25" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C25" s="35" t="n">
+        <x:v>46285</x:v>
+      </x:c>
+      <x:c r="D25" s="34" t="str">
+        <x:v>feat: 未发布草稿可由管理员立即永久删除（带原因与审计）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record the dept-head reader account (deployment data change)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R0744ae9eeb534ce3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rc21168e7e9cd4c9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R7488e54e31b84a28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R94ab8c1fd9654151"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R0c3e71efa21a4d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R49be0552c0b04819"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -899,23 +899,43 @@
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="33" t="str">
+      <x:c r="A26" s="29" t="str">
         <x:v>V3.5</x:v>
       </x:c>
-      <x:c r="B26" s="35" t="n">
+      <x:c r="B26" s="31" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="C26" s="34" t="str">
-        <x:v>小型修改</x:v>
-      </x:c>
-      <x:c r="D26" s="34" t="str">
+      <x:c r="C26" s="30" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D26" s="30" t="str">
         <x:v>按用户确认放宽永久清理规则：从未发布过的草稿可由管理员在回收站立即永久删除，删除必须填写原因并写入审计（规则标记 never-published-draft）；已发布过的内容仍保留 30 天才能清理，避免读者侧内容被误删。回收站列表对可立即删除的条目显示原因提示与删除原因输入框，删除失败改为错误提示；同步更新需求文档 DEL-02、验收准则与 CONTEXT 的措辞</x:v>
       </x:c>
-      <x:c r="E26" s="34" t="str">
+      <x:c r="E26" s="30" t="str">
         <x:v>本次提交，标签 v3.5</x:v>
       </x:c>
-      <x:c r="F26" s="34" t="str">
+      <x:c r="F26" s="30" t="str">
         <x:v>模块用例覆盖：未发布草稿可立即删除且写审计（含 rule 字段）、空白原因被拒、已发布内容仍报「保留 30 天」；e2e 覆盖编辑者归档→管理员带原因永久删除→列表与阅读侧彻底消失；全量 283 单元用例、9 个 PostgreSQL 容器用例、86 条 e2e 通过；线上实测完整走通一次（含审计留痕）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="33" t="str">
+        <x:v>V3.5</x:v>
+      </x:c>
+      <x:c r="B27" s="35" t="n">
+        <x:v>46285</x:v>
+      </x:c>
+      <x:c r="C27" s="34" t="str">
+        <x:v>数据变更</x:v>
+      </x:c>
+      <x:c r="D27" s="34" t="str">
+        <x:v>部署库新增阅读者账号 dept-head（显示名「部门长」），用于部门长阅读测试；账号按 AUTH-01 由管理员在后台创建，不带自助注册，首登强制改密（AUTH-02）</x:v>
+      </x:c>
+      <x:c r="E27" s="34" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F27" s="34" t="str">
+        <x:v>管理员后台创建成功并写入审计（account-creation, role=reader）；实测首次登录进入「设置你的正式密码」页；账号列表显示「部门长 @dept-head 阅读者 已启用」；验证用会话已注销</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: allow admins to change usernames and display names (V3.6)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R94ab8c1fd9654151"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R0c3e71efa21a4d6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R49be0552c0b04819"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R11d8baf327f8447e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R79b3546235864ee3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Re87e6de251584881"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -919,23 +919,43 @@
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="33" t="str">
+      <x:c r="A27" s="29" t="str">
         <x:v>V3.5</x:v>
       </x:c>
-      <x:c r="B27" s="35" t="n">
+      <x:c r="B27" s="31" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="C27" s="34" t="str">
+      <x:c r="C27" s="30" t="str">
         <x:v>数据变更</x:v>
       </x:c>
-      <x:c r="D27" s="34" t="str">
+      <x:c r="D27" s="30" t="str">
         <x:v>部署库新增阅读者账号 dept-head（显示名「部门长」），用于部门长阅读测试；账号按 AUTH-01 由管理员在后台创建，不带自助注册，首登强制改密（AUTH-02）</x:v>
       </x:c>
-      <x:c r="E27" s="34" t="str">
+      <x:c r="E27" s="30" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="F27" s="34" t="str">
+      <x:c r="F27" s="30" t="str">
         <x:v>管理员后台创建成功并写入审计（account-creation, role=reader）；实测首次登录进入「设置你的正式密码」页；账号列表显示「部门长 @dept-head 阅读者 已启用」；验证用会话已注销</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="33" t="str">
+        <x:v>V3.6</x:v>
+      </x:c>
+      <x:c r="B28" s="35" t="n">
+        <x:v>46285</x:v>
+      </x:c>
+      <x:c r="C28" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D28" s="34" t="str">
+        <x:v>账户管理新增「修改用户名与显示名称」：管理员可在成员卡片上直接改用户名与显示名称（不改密码、不改角色），改动写入身份审计 account-identity-update（含改前/改后用户名与显示名称）；用户名大小写不敏感唯一，空值与重名被拒，阅读者伪造调用被拒</x:v>
+      </x:c>
+      <x:c r="E28" s="34" t="str">
+        <x:v>本次提交，标签 v3.6</x:v>
+      </x:c>
+      <x:c r="F28" s="34" t="str">
+        <x:v>模块用例：改名后旧用户名登录失败、新用户名沿用原密码可登录并进入首登改密、审计含前后值、重名与空值被拒、阅读者被拒；e2e：管理员后台改名后列表显示新用户名与显示名、旧用户名不可登录；全量 285 单元用例、9 个 PostgreSQL 容器用例、87 条 e2e 通过</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1267,17 +1287,31 @@
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="33" t="str">
+      <x:c r="A25" s="29" t="str">
         <x:v>V3.5</x:v>
       </x:c>
-      <x:c r="B25" s="34" t="str">
+      <x:c r="B25" s="30" t="str">
         <x:v>（本次提交）</x:v>
       </x:c>
-      <x:c r="C25" s="35" t="n">
+      <x:c r="C25" s="31" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="D25" s="34" t="str">
+      <x:c r="D25" s="30" t="str">
         <x:v>feat: 未发布草稿可由管理员立即永久删除（带原因与审计）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="33" t="str">
+        <x:v>V3.6</x:v>
+      </x:c>
+      <x:c r="B26" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C26" s="35" t="n">
+        <x:v>46285</x:v>
+      </x:c>
+      <x:c r="D26" s="34" t="str">
+        <x:v>feat: 账户管理支持修改用户名与显示名称（带审计）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record the Lou rename and 10 department-head reader accounts
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R11d8baf327f8447e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R79b3546235864ee3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Re87e6de251584881"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rb67bfef626144aae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rd0bd752a08904f6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rbacc2fffa07f4484"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -939,23 +939,43 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="33" t="str">
+      <x:c r="A28" s="29" t="str">
         <x:v>V3.6</x:v>
       </x:c>
-      <x:c r="B28" s="35" t="n">
+      <x:c r="B28" s="31" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="C28" s="34" t="str">
-        <x:v>小型修改</x:v>
-      </x:c>
-      <x:c r="D28" s="34" t="str">
+      <x:c r="C28" s="30" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D28" s="30" t="str">
         <x:v>账户管理新增「修改用户名与显示名称」：管理员可在成员卡片上直接改用户名与显示名称（不改密码、不改角色），改动写入身份审计 account-identity-update（含改前/改后用户名与显示名称）；用户名大小写不敏感唯一，空值与重名被拒，阅读者伪造调用被拒</x:v>
       </x:c>
-      <x:c r="E28" s="34" t="str">
+      <x:c r="E28" s="30" t="str">
         <x:v>本次提交，标签 v3.6</x:v>
       </x:c>
-      <x:c r="F28" s="34" t="str">
+      <x:c r="F28" s="30" t="str">
         <x:v>模块用例：改名后旧用户名登录失败、新用户名沿用原密码可登录并进入首登改密、审计含前后值、重名与空值被拒、阅读者被拒；e2e：管理员后台改名后列表显示新用户名与显示名、旧用户名不可登录；全量 285 单元用例、9 个 PostgreSQL 容器用例、87 条 e2e 通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="33" t="str">
+        <x:v>V3.6</x:v>
+      </x:c>
+      <x:c r="B29" s="35" t="n">
+        <x:v>46285</x:v>
+      </x:c>
+      <x:c r="C29" s="34" t="str">
+        <x:v>数据变更</x:v>
+      </x:c>
+      <x:c r="D29" s="34" t="str">
+        <x:v>管理员账号 qadmin 改名为 Lou（密码不变，审计 account-identity-update 记录 previousUsername=qadmin）；新增 10 个部门长阅读账号 Nancy / Ivy / Harris / EZ / Kevin / Reina / Allan / Dennis / Claire / Wayde，统一初始密码，均要求首次登录改为自己的密码</x:v>
+      </x:c>
+      <x:c r="E29" s="34" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F29" s="34" t="str">
+        <x:v>后台改名成功并留审计；10 个账号创建成功（account-creation, role=reader）且状态为已启用、待首登改密；实测 Nancy、Wayde 首次登录均进入「设置你的正式密码」页；验证用会话已注销</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
style: greeting on one line, login title split zh/en (V3.7)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rb67bfef626144aae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rd0bd752a08904f6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rbacc2fffa07f4484"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rda305571fde14a35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R44cbe284a1c147ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R5dbaf860edd447b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -959,23 +959,43 @@
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="33" t="str">
+      <x:c r="A29" s="29" t="str">
         <x:v>V3.6</x:v>
       </x:c>
-      <x:c r="B29" s="35" t="n">
+      <x:c r="B29" s="31" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="C29" s="34" t="str">
+      <x:c r="C29" s="30" t="str">
         <x:v>数据变更</x:v>
       </x:c>
-      <x:c r="D29" s="34" t="str">
+      <x:c r="D29" s="30" t="str">
         <x:v>管理员账号 qadmin 改名为 Lou（密码不变，审计 account-identity-update 记录 previousUsername=qadmin）；新增 10 个部门长阅读账号 Nancy / Ivy / Harris / EZ / Kevin / Reina / Allan / Dennis / Claire / Wayde，统一初始密码，均要求首次登录改为自己的密码</x:v>
       </x:c>
-      <x:c r="E29" s="34" t="str">
+      <x:c r="E29" s="30" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="F29" s="34" t="str">
+      <x:c r="F29" s="30" t="str">
         <x:v>后台改名成功并留审计；10 个账号创建成功（account-creation, role=reader）且状态为已启用、待首登改密；实测 Nancy、Wayde 首次登录均进入「设置你的正式密码」页；验证用会话已注销</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="33" t="str">
+        <x:v>V3.7</x:v>
+      </x:c>
+      <x:c r="B30" s="35" t="n">
+        <x:v>46285</x:v>
+      </x:c>
+      <x:c r="C30" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D30" s="34" t="str">
+        <x:v>两处排版调整（用户反馈）：① 首页问候由「问候小字一行 + 名字一行」改为「名字 + 问候语」同一行、同一字号（如「Lou 下午好」），名字与问候各自不可拆开；② 登录页标题改为中文一行（登录品集｜）、英文一行（Q Nexus），避免在 Q 与 Nexus 之间断行；两处字号按视口收敛，390px 窄屏与 200% 缩放均不产生横向滚动</x:v>
+      </x:c>
+      <x:c r="E30" s="34" t="str">
+        <x:v>本次提交，标签 v3.7</x:v>
+      </x:c>
+      <x:c r="F30" s="34" t="str">
+        <x:v>e2e 新增断言：首页问候文字为「显示名 + 问候语」且两部分顶边一致（同一行）且字号一致，390px 仍同一行且无横向滚动；登录页标题为两行、Q Nexus 不拆行；全量 285 单元用例、9 个 PostgreSQL 容器用例、87 条 e2e 通过</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1321,17 +1341,31 @@
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="33" t="str">
+      <x:c r="A26" s="29" t="str">
         <x:v>V3.6</x:v>
       </x:c>
-      <x:c r="B26" s="34" t="str">
+      <x:c r="B26" s="30" t="str">
         <x:v>（本次提交）</x:v>
       </x:c>
-      <x:c r="C26" s="35" t="n">
+      <x:c r="C26" s="31" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="D26" s="34" t="str">
+      <x:c r="D26" s="30" t="str">
         <x:v>feat: 账户管理支持修改用户名与显示名称（带审计）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="33" t="str">
+        <x:v>V3.7</x:v>
+      </x:c>
+      <x:c r="B27" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C27" s="35" t="n">
+        <x:v>46285</x:v>
+      </x:c>
+      <x:c r="D27" s="34" t="str">
+        <x:v>style: 首页问候同行同字号、登录标题中英分行</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix: readers could not open any article on PostgreSQL (V3.8)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rda305571fde14a35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R44cbe284a1c147ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R5dbaf860edd447b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Re8dc17c14163419a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Read3e0043f0644ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R16f37578b20b4b27"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -979,23 +979,43 @@
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="33" t="str">
+      <x:c r="A30" s="29" t="str">
         <x:v>V3.7</x:v>
       </x:c>
-      <x:c r="B30" s="35" t="n">
+      <x:c r="B30" s="31" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="C30" s="34" t="str">
-        <x:v>小型修改</x:v>
-      </x:c>
-      <x:c r="D30" s="34" t="str">
+      <x:c r="C30" s="30" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D30" s="30" t="str">
         <x:v>两处排版调整（用户反馈）：① 首页问候由「问候小字一行 + 名字一行」改为「名字 + 问候语」同一行、同一字号（如「Lou 下午好」），名字与问候各自不可拆开；② 登录页标题改为中文一行（登录品集｜）、英文一行（Q Nexus），避免在 Q 与 Nexus 之间断行；两处字号按视口收敛，390px 窄屏与 200% 缩放均不产生横向滚动</x:v>
       </x:c>
-      <x:c r="E30" s="34" t="str">
+      <x:c r="E30" s="30" t="str">
         <x:v>本次提交，标签 v3.7</x:v>
       </x:c>
-      <x:c r="F30" s="34" t="str">
+      <x:c r="F30" s="30" t="str">
         <x:v>e2e 新增断言：首页问候文字为「显示名 + 问候语」且两部分顶边一致（同一行）且字号一致，390px 仍同一行且无横向滚动；登录页标题为两行、Q Nexus 不拆行；全量 285 单元用例、9 个 PostgreSQL 容器用例、87 条 e2e 通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="33" t="str">
+        <x:v>V3.8</x:v>
+      </x:c>
+      <x:c r="B31" s="35" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="C31" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D31" s="34" t="str">
+        <x:v>修复「阅读者身份在新人专区/知识页点不进任何文章」：根因是 content-stats 的阅读计数把 Date 直接插进 drizzle 的 sql 模板，PGlite（自动化测试用的引擎）能容忍，线上 postgres.js 驱动在参数编码时抛 ERR_INVALID_ARG_TYPE；该代码路径只在非编辑/管理员（阅读者）访问文章时执行，因此管理员打开正常、阅读者必然 500（点击后停在原页）。改为使用类型化操作符 lt/gte（子查询别名处传 ISO 字符串），同文件里统计看板、待复核列表与身份明细清理的同类写法一并修复</x:v>
+      </x:c>
+      <x:c r="E31" s="34" t="str">
+        <x:v>本次提交，标签 v3.8</x:v>
+      </x:c>
+      <x:c r="F31" s="34" t="str">
+        <x:v>新增真实 PostgreSQL 集成用例（tests/integration/content-stats-postgresql.test.ts）：阅读计数、统计看板日期聚合、保留期清理三条路径；回退修复时该用例报出与线上一致的 ERR_INVALID_ARG_TYPE，说明能挡住同类回归；全量 285 单元用例、12 个 PostgreSQL 容器用例、87 条 e2e 通过；线上以阅读者身份实测新人专区文章可正常打开</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1355,17 +1375,31 @@
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="33" t="str">
+      <x:c r="A27" s="29" t="str">
         <x:v>V3.7</x:v>
       </x:c>
-      <x:c r="B27" s="34" t="str">
+      <x:c r="B27" s="30" t="str">
         <x:v>（本次提交）</x:v>
       </x:c>
-      <x:c r="C27" s="35" t="n">
+      <x:c r="C27" s="31" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="D27" s="34" t="str">
+      <x:c r="D27" s="30" t="str">
         <x:v>style: 首页问候同行同字号、登录标题中英分行</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="33" t="str">
+        <x:v>V3.8</x:v>
+      </x:c>
+      <x:c r="B28" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C28" s="35" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="D28" s="34" t="str">
+        <x:v>fix: 阅读者打不开文章（sql 模板裸 Date 导致 postgres.js 参数编码失败）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix: callout styles hit rendered HTML, preview reuses ArticleBody, properties open by default, code block command (V3.9)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Re8dc17c14163419a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Read3e0043f0644ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R16f37578b20b4b27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R6535681fd9c24cd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R47137c9e6d4e435b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R86893b030bad439e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -999,23 +999,43 @@
       </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="33" t="str">
+      <x:c r="A31" s="29" t="str">
         <x:v>V3.8</x:v>
       </x:c>
-      <x:c r="B31" s="35" t="n">
+      <x:c r="B31" s="31" t="n">
         <x:v>46286</x:v>
       </x:c>
-      <x:c r="C31" s="34" t="str">
-        <x:v>小型修改</x:v>
-      </x:c>
-      <x:c r="D31" s="34" t="str">
+      <x:c r="C31" s="30" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D31" s="30" t="str">
         <x:v>修复「阅读者身份在新人专区/知识页点不进任何文章」：根因是 content-stats 的阅读计数把 Date 直接插进 drizzle 的 sql 模板，PGlite（自动化测试用的引擎）能容忍，线上 postgres.js 驱动在参数编码时抛 ERR_INVALID_ARG_TYPE；该代码路径只在非编辑/管理员（阅读者）访问文章时执行，因此管理员打开正常、阅读者必然 500（点击后停在原页）。改为使用类型化操作符 lt/gte（子查询别名处传 ISO 字符串），同文件里统计看板、待复核列表与身份明细清理的同类写法一并修复</x:v>
       </x:c>
-      <x:c r="E31" s="34" t="str">
+      <x:c r="E31" s="30" t="str">
         <x:v>本次提交，标签 v3.8</x:v>
       </x:c>
-      <x:c r="F31" s="34" t="str">
+      <x:c r="F31" s="30" t="str">
         <x:v>新增真实 PostgreSQL 集成用例（tests/integration/content-stats-postgresql.test.ts）：阅读计数、统计看板日期聚合、保留期清理三条路径；回退修复时该用例报出与线上一致的 ERR_INVALID_ARG_TYPE，说明能挡住同类回归；全量 285 单元用例、12 个 PostgreSQL 容器用例、87 条 e2e 通过；线上以阅读者身份实测新人专区文章可正常打开</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="33" t="str">
+        <x:v>V3.9</x:v>
+      </x:c>
+      <x:c r="B32" s="35" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="C32" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D32" s="34" t="str">
+        <x:v>编辑器与正文四处修复（用户反馈）：① Callout / 公式排版失效——CSS Modules 把 article-body.module.css 里针对渲染产物的 .callout*、.callout-icon、.katex-display 类名一并哈希，而 Markdown 渲染出的 HTML 用原始类名，选择器永远匹配不上，Callout 退化成普通段落（阅读页与主题页内联正文同时受益）；② 编辑器预览区没有正文排版容器，预览里 callout / 代码块 / 标题都没有样式，改为复用与阅读页相同的 ArticleBody 组件；③ 属性面板默认展开，面板内新增「收起」，工具栏「属性」改为幂等展开；④ 命令菜单新增「代码块」，一键插入围栏代码块，避免手打成两个反引号而不生效</x:v>
+      </x:c>
+      <x:c r="E32" s="34" t="str">
+        <x:v>本次提交，标签 v3.9</x:v>
+      </x:c>
+      <x:c r="F32" s="34" t="str">
+        <x:v>e2e 新增断言：阅读页与编辑器预览的 Callout 必须命中样式（padding-left 16px、border-left 3px、图标 ::before 显示「重点」）——修复前预览处 padding-left 为 0px；编辑器用例断言属性面板默认可见、可收起再展开；模块用例新增代码块命令；全量 286 单元用例、12 个 PostgreSQL 容器用例、87 条 e2e 通过；线上用编辑者身份实测阅读页与预览均正常</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1389,17 +1409,31 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="33" t="str">
+      <x:c r="A28" s="29" t="str">
         <x:v>V3.8</x:v>
       </x:c>
-      <x:c r="B28" s="34" t="str">
+      <x:c r="B28" s="30" t="str">
         <x:v>（本次提交）</x:v>
       </x:c>
-      <x:c r="C28" s="35" t="n">
+      <x:c r="C28" s="31" t="n">
         <x:v>46286</x:v>
       </x:c>
-      <x:c r="D28" s="34" t="str">
+      <x:c r="D28" s="30" t="str">
         <x:v>fix: 阅读者打不开文章（sql 模板裸 Date 导致 postgres.js 参数编码失败）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="33" t="str">
+        <x:v>V3.9</x:v>
+      </x:c>
+      <x:c r="B29" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C29" s="35" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="D29" s="34" t="str">
+        <x:v>fix: Callout 样式命中（:global）、预览复用 ArticleBody、属性面板默认展开、新增代码块命令</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
style: callout redesign without text labels (V3.10)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R6535681fd9c24cd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R47137c9e6d4e435b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R86893b030bad439e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R08e9496c9e28443d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rdcb4b4f78e484cfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rf02deac5fad34eec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1019,23 +1019,43 @@
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="33" t="str">
+      <x:c r="A32" s="29" t="str">
         <x:v>V3.9</x:v>
       </x:c>
-      <x:c r="B32" s="35" t="n">
+      <x:c r="B32" s="31" t="n">
         <x:v>46286</x:v>
       </x:c>
-      <x:c r="C32" s="34" t="str">
-        <x:v>小型修改</x:v>
-      </x:c>
-      <x:c r="D32" s="34" t="str">
+      <x:c r="C32" s="30" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D32" s="30" t="str">
         <x:v>编辑器与正文四处修复（用户反馈）：① Callout / 公式排版失效——CSS Modules 把 article-body.module.css 里针对渲染产物的 .callout*、.callout-icon、.katex-display 类名一并哈希，而 Markdown 渲染出的 HTML 用原始类名，选择器永远匹配不上，Callout 退化成普通段落（阅读页与主题页内联正文同时受益）；② 编辑器预览区没有正文排版容器，预览里 callout / 代码块 / 标题都没有样式，改为复用与阅读页相同的 ArticleBody 组件；③ 属性面板默认展开，面板内新增「收起」，工具栏「属性」改为幂等展开；④ 命令菜单新增「代码块」，一键插入围栏代码块，避免手打成两个反引号而不生效</x:v>
       </x:c>
-      <x:c r="E32" s="34" t="str">
+      <x:c r="E32" s="30" t="str">
         <x:v>本次提交，标签 v3.9</x:v>
       </x:c>
-      <x:c r="F32" s="34" t="str">
+      <x:c r="F32" s="30" t="str">
         <x:v>e2e 新增断言：阅读页与编辑器预览的 Callout 必须命中样式（padding-left 16px、border-left 3px、图标 ::before 显示「重点」）——修复前预览处 padding-left 为 0px；编辑器用例断言属性面板默认可见、可收起再展开；模块用例新增代码块命令；全量 286 单元用例、12 个 PostgreSQL 容器用例、87 条 e2e 通过；线上用编辑者身份实测阅读页与预览均正常</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="33" t="str">
+        <x:v>V3.10</x:v>
+      </x:c>
+      <x:c r="B33" s="35" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="C33" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D33" s="34" t="str">
+        <x:v>Callout 视觉改版（用户确认方案 A「左侧色条 + 极淡同色底 + 标题同色」）：不再显示「信息 / 提示 / 重点 / 警告 / 示例 / 公式」文字标签；六种类型分别用左侧 4px 色条 + 极淡同色底 + 同色加粗标题区分，正文保持正常文字色；强调色与底色在浅色 / 深色 / 跟随系统三种主题下分别取值，新增 --callout-* 设计令牌（tokens.css）；类型名保留在无障碍层（仅屏幕阅读器可见）以免读屏用户丢失语义；同步更新视觉规范 §9 的类型样式表与「不再用文字标签」的决定</x:v>
+      </x:c>
+      <x:c r="E33" s="34" t="str">
+        <x:v>本次提交，标签 v3.10</x:v>
+      </x:c>
+      <x:c r="F33" s="34" t="str">
+        <x:v>e2e 断言更新为：Callout 左侧色条 4px、标题使用类型色、类型名仍可被读屏读取但视觉上被裁掉（clip-path）；浅色与深色主题分别截图核对（左侧色条 + 淡色底 + 同色标题，无文字标签）；全量 286 单元用例、12 个 PostgreSQL 容器用例、87 条 e2e 通过；线上用编辑者身份实测阅读页与编辑器预览一致</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1423,17 +1443,31 @@
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="33" t="str">
+      <x:c r="A29" s="29" t="str">
         <x:v>V3.9</x:v>
       </x:c>
-      <x:c r="B29" s="34" t="str">
+      <x:c r="B29" s="30" t="str">
         <x:v>（本次提交）</x:v>
       </x:c>
-      <x:c r="C29" s="35" t="n">
+      <x:c r="C29" s="31" t="n">
         <x:v>46286</x:v>
       </x:c>
-      <x:c r="D29" s="34" t="str">
+      <x:c r="D29" s="30" t="str">
         <x:v>fix: Callout 样式命中（:global）、预览复用 ArticleBody、属性面板默认展开、新增代码块命令</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="33" t="str">
+        <x:v>V3.10</x:v>
+      </x:c>
+      <x:c r="B30" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C30" s="35" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="D30" s="34" t="str">
+        <x:v>style: Callout 去掉文字标签，改用类型色条 + 淡底 + 同色标题（方案 A）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
style: muted callout palette with bar/tint/edge (V3.11)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R08e9496c9e28443d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rdcb4b4f78e484cfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rf02deac5fad34eec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rf506c68942f04105"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R9f88722491144780"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R55109bd3e5b2423b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1039,23 +1039,43 @@
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="33" t="str">
+      <x:c r="A33" s="29" t="str">
         <x:v>V3.10</x:v>
       </x:c>
-      <x:c r="B33" s="35" t="n">
+      <x:c r="B33" s="31" t="n">
         <x:v>46286</x:v>
       </x:c>
-      <x:c r="C33" s="34" t="str">
-        <x:v>小型修改</x:v>
-      </x:c>
-      <x:c r="D33" s="34" t="str">
+      <x:c r="C33" s="30" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D33" s="30" t="str">
         <x:v>Callout 视觉改版（用户确认方案 A「左侧色条 + 极淡同色底 + 标题同色」）：不再显示「信息 / 提示 / 重点 / 警告 / 示例 / 公式」文字标签；六种类型分别用左侧 4px 色条 + 极淡同色底 + 同色加粗标题区分，正文保持正常文字色；强调色与底色在浅色 / 深色 / 跟随系统三种主题下分别取值，新增 --callout-* 设计令牌（tokens.css）；类型名保留在无障碍层（仅屏幕阅读器可见）以免读屏用户丢失语义；同步更新视觉规范 §9 的类型样式表与「不再用文字标签」的决定</x:v>
       </x:c>
-      <x:c r="E33" s="34" t="str">
+      <x:c r="E33" s="30" t="str">
         <x:v>本次提交，标签 v3.10</x:v>
       </x:c>
-      <x:c r="F33" s="34" t="str">
+      <x:c r="F33" s="30" t="str">
         <x:v>e2e 断言更新为：Callout 左侧色条 4px、标题使用类型色、类型名仍可被读屏读取但视觉上被裁掉（clip-path）；浅色与深色主题分别截图核对（左侧色条 + 淡色底 + 同色标题，无文字标签）；全量 286 单元用例、12 个 PostgreSQL 容器用例、87 条 e2e 通过；线上用编辑者身份实测阅读页与编辑器预览一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="33" t="str">
+        <x:v>V3.11</x:v>
+      </x:c>
+      <x:c r="B34" s="35" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="C34" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D34" s="34" t="str">
+        <x:v>Callout 配色重做（用户反馈上一版配色偏「廉价」，确认采用方案 2）：把六个高饱和类型色换成同一明度、低饱和的一组（石墨蓝 #5F7186 / 苔绿 #55715A / 靛蓝 #2F6FBA / 赭石 #9A6B2F / 灰紫 #6F6291 / 灰青 #437B76，深色主题另取一组更亮的同族色）；结构改为左侧 4px 类型色条 + 5% 同色底 + 1px 同色细描边 + 右侧 8px 圆角 + 同色标题，正文保持正常文字色；底色与描边为精确混色值（不依赖 color-mix），写入 tokens.css 的 --callout-* 令牌，覆盖浅色 / 深色 / 跟随系统三种主题；视觉规范 §9 类型配色表同步更新</x:v>
+      </x:c>
+      <x:c r="E34" s="34" t="str">
+        <x:v>本次提交，标签 v3.11</x:v>
+      </x:c>
+      <x:c r="F34" s="34" t="str">
+        <x:v>先出可视化设计稿（浅色 + 深色，六种类型并排）供确认后再改代码；e2e 断言更新为：色条 4px、标题使用类型色 rgb(47,111,186)、底色 rgb(245,248,252)、细描边 1px、类型名仅读屏可见；全量 286 单元用例、12 个 PostgreSQL 容器用例、87 条 e2e 通过；本地与线上各截浅色 / 深色核对，发布过的文章刷新即生效无需重发</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1457,17 +1477,31 @@
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="33" t="str">
+      <x:c r="A30" s="29" t="str">
         <x:v>V3.10</x:v>
       </x:c>
-      <x:c r="B30" s="34" t="str">
-        <x:v>（本次提交）</x:v>
-      </x:c>
-      <x:c r="C30" s="35" t="n">
+      <x:c r="B30" s="30" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C30" s="31" t="n">
         <x:v>46286</x:v>
       </x:c>
-      <x:c r="D30" s="34" t="str">
+      <x:c r="D30" s="30" t="str">
         <x:v>style: Callout 去掉文字标签，改用类型色条 + 淡底 + 同色标题（方案 A）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="33" t="str">
+        <x:v>V3.11</x:v>
+      </x:c>
+      <x:c r="B31" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C31" s="35" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="D31" s="34" t="str">
+        <x:v>style: Callout 配色重做（低饱和同明度 + 色条/淡底/细描边）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
style: callouts default to bold (V3.12)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rf506c68942f04105"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R9f88722491144780"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R55109bd3e5b2423b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R7f5ff7d5c4bc47f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R5cfb24305d02499d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R24a799dce3264329"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1059,23 +1059,43 @@
       </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="33" t="str">
+      <x:c r="A34" s="29" t="str">
         <x:v>V3.11</x:v>
       </x:c>
-      <x:c r="B34" s="35" t="n">
+      <x:c r="B34" s="31" t="n">
         <x:v>46286</x:v>
       </x:c>
-      <x:c r="C34" s="34" t="str">
-        <x:v>小型修改</x:v>
-      </x:c>
-      <x:c r="D34" s="34" t="str">
+      <x:c r="C34" s="30" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D34" s="30" t="str">
         <x:v>Callout 配色重做（用户反馈上一版配色偏「廉价」，确认采用方案 2）：把六个高饱和类型色换成同一明度、低饱和的一组（石墨蓝 #5F7186 / 苔绿 #55715A / 靛蓝 #2F6FBA / 赭石 #9A6B2F / 灰紫 #6F6291 / 灰青 #437B76，深色主题另取一组更亮的同族色）；结构改为左侧 4px 类型色条 + 5% 同色底 + 1px 同色细描边 + 右侧 8px 圆角 + 同色标题，正文保持正常文字色；底色与描边为精确混色值（不依赖 color-mix），写入 tokens.css 的 --callout-* 令牌，覆盖浅色 / 深色 / 跟随系统三种主题；视觉规范 §9 类型配色表同步更新</x:v>
       </x:c>
-      <x:c r="E34" s="34" t="str">
+      <x:c r="E34" s="30" t="str">
         <x:v>本次提交，标签 v3.11</x:v>
       </x:c>
-      <x:c r="F34" s="34" t="str">
+      <x:c r="F34" s="30" t="str">
         <x:v>先出可视化设计稿（浅色 + 深色，六种类型并排）供确认后再改代码；e2e 断言更新为：色条 4px、标题使用类型色 rgb(47,111,186)、底色 rgb(245,248,252)、细描边 1px、类型名仅读屏可见；全量 286 单元用例、12 个 PostgreSQL 容器用例、87 条 e2e 通过；本地与线上各截浅色 / 深色核对，发布过的文章刷新即生效无需重发</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="33" t="str">
+        <x:v>V3.12</x:v>
+      </x:c>
+      <x:c r="B35" s="35" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="C35" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D35" s="34" t="str">
+        <x:v>Callout 内容默认加粗（用户要求「所有 callout 都设置成粗体」）：在 .callout 上设置 font-weight: 700，标题、正文、列表项一并加粗，与正文形成明显对比；标题仍通过类型色区分，不再靠字重；公式（KaTeX 自带字重）与代码块同样继承加粗；视觉规范 §9 增加「Callout 默认加粗」约定</x:v>
+      </x:c>
+      <x:c r="E35" s="34" t="str">
+        <x:v>本次提交，标签 v3.12</x:v>
+      </x:c>
+      <x:c r="F35" s="34" t="str">
+        <x:v>e2e 断言新增：Callout 容器与内部正文段落计算字重均为 700（修复前正文为 400，断言先红后绿）；同时核对含列表、代码块、公式的复合 Callout 在浅色 / 深色下的可读性；全量 286 单元用例、12 个 PostgreSQL 容器用例、87 条 e2e 通过；线上实测阅读页与编辑器预览一致</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1491,17 +1511,31 @@
       </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="33" t="str">
+      <x:c r="A31" s="29" t="str">
         <x:v>V3.11</x:v>
       </x:c>
-      <x:c r="B31" s="34" t="str">
-        <x:v>（本次提交）</x:v>
-      </x:c>
-      <x:c r="C31" s="35" t="n">
+      <x:c r="B31" s="30" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C31" s="31" t="n">
         <x:v>46286</x:v>
       </x:c>
-      <x:c r="D31" s="34" t="str">
+      <x:c r="D31" s="30" t="str">
         <x:v>style: Callout 配色重做（低饱和同明度 + 色条/淡底/细描边）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="33" t="str">
+        <x:v>V3.12</x:v>
+      </x:c>
+      <x:c r="B32" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C32" s="35" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="D32" s="34" t="str">
+        <x:v>style: Callout 内容默认加粗（font-weight 700）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record V3.13 change log
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R7f5ff7d5c4bc47f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R5cfb24305d02499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R24a799dce3264329"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R67f54527c08d437b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R1df797a54d70481b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rba39bf7838994986"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1098,6 +1098,26 @@
         <x:v>e2e 断言新增：Callout 容器与内部正文段落计算字重均为 700（修复前正文为 400，断言先红后绿）；同时核对含列表、代码块、公式的复合 Callout 在浅色 / 深色下的可读性；全量 286 单元用例、12 个 PostgreSQL 容器用例、87 条 e2e 通过；线上实测阅读页与编辑器预览一致</x:v>
       </x:c>
     </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>V3.13</x:v>
+      </x:c>
+      <x:c r="B36" s="3" t="n">
+        <x:v>46288</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>登录页与首页视觉精修：重排登录表单并增加密码显隐；统一动效令牌与减弱动态效果；首页搜索增加 Ctrl/⌘ K、焦点圈定和视口级浮层；内容区块增加克制的入场、图形揭示和悬停反馈。</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>133090b, 标签 v3.13</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
+        <x:v>Playwright 关键页面 13 项通过；typecheck、lint、format、单元测试与 production build 通过；登录页、首页和搜索浮层已人工检查。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1538,6 +1558,20 @@
         <x:v>style: Callout 内容默认加粗（font-weight 700）</x:v>
       </x:c>
     </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>V3.13</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>133090b</x:v>
+      </x:c>
+      <x:c r="C33" s="3" t="n">
+        <x:v>46288</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>style: 登录页与首页动效及高级感精修</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix: make backup and restore verification complete (V3.14)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R67f54527c08d437b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R1df797a54d70481b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rba39bf7838994986"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Red1dbadfe72846b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rc1dc9b6b94eb42b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R9ef434d6c1b14e42"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1109,13 +1109,33 @@
         <x:v>小型修改</x:v>
       </x:c>
       <x:c r="D36" t="str">
-        <x:v>登录页与首页视觉精修：重排登录表单并增加密码显隐；统一动效令牌与减弱动态效果；首页搜索增加 Ctrl/⌘ K、焦点圈定和视口级浮层；内容区块增加克制的入场、图形揭示和悬停反馈。</x:v>
+        <x:v>登录页与首页视觉精修：重排登录表单并增加密码显隐；统一动效令牌与减弱动态效果；首页搜索补充快捷键、焦点圈定和视口级浮层；内容区块增加克制的入场、图形揭示和悬停反馈</x:v>
       </x:c>
       <x:c r="E36" t="str">
-        <x:v>133090b, 标签 v3.13</x:v>
+        <x:v>标签 v3.13</x:v>
       </x:c>
       <x:c r="F36" t="str">
-        <x:v>Playwright 关键页面 13 项通过；typecheck、lint、format、单元测试与 production build 通过；登录页、首页和搜索浮层已人工检查。</x:v>
+        <x:v>登录与首页相关 E2E、typecheck、build 通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>V3.14</x:v>
+      </x:c>
+      <x:c r="B37" s="3" t="n">
+        <x:v>46288</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>修复备份与恢复不可验证：手工备份强制包含非空 PostgreSQL 转储和上传文件；后台显示配置状态并支持完整性验证；Compose 初始化备份目录并内置数据库工具；新增隔离数据库恢复演练与审计</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>标签 v3.14</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>备份模块测试、后台 E2E、Compose 配置契约与真实容器备份—隔离恢复闭环通过</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1563,13 +1583,27 @@
         <x:v>V3.13</x:v>
       </x:c>
       <x:c r="B33" t="str">
-        <x:v>133090b</x:v>
+        <x:v>（本次提交）</x:v>
       </x:c>
       <x:c r="C33" s="3" t="n">
         <x:v>46288</x:v>
       </x:c>
       <x:c r="D33" t="str">
-        <x:v>style: 登录页与首页动效及高级感精修</x:v>
+        <x:v>style: 登录页与首页交互动效精修</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>V3.14</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C34" s="3" t="n">
+        <x:v>46288</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>fix: 完整备份与隔离数据库恢复演练</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record the local deployment to V3.14
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Red1dbadfe72846b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rc1dc9b6b94eb42b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R9ef434d6c1b14e42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R0da48958d4fe4859"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Re3f7256d6ef24e91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R7f43535eba5f4e96"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -149,7 +149,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="43">
+  <x:cellXfs count="44">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -233,6 +233,7 @@
     <x:xf numFmtId="0" fontId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1119,23 +1120,43 @@
       </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" t="str">
+      <x:c r="A37" s="26" t="str">
         <x:v>V3.14</x:v>
       </x:c>
-      <x:c r="B37" s="3" t="n">
+      <x:c r="B37" s="43" t="n">
         <x:v>46288</x:v>
       </x:c>
-      <x:c r="C37" t="str">
-        <x:v>小型修改</x:v>
-      </x:c>
-      <x:c r="D37" t="str">
+      <x:c r="C37" s="27" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D37" s="27" t="str">
         <x:v>修复备份与恢复不可验证：手工备份强制包含非空 PostgreSQL 转储和上传文件；后台显示配置状态并支持完整性验证；Compose 初始化备份目录并内置数据库工具；新增隔离数据库恢复演练与审计</x:v>
       </x:c>
-      <x:c r="E37" t="str">
+      <x:c r="E37" s="27" t="str">
         <x:v>标签 v3.14</x:v>
       </x:c>
-      <x:c r="F37" t="str">
+      <x:c r="F37" s="28" t="str">
         <x:v>备份模块测试、后台 E2E、Compose 配置契约与真实容器备份—隔离恢复闭环通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="33" t="str">
+        <x:v>V3.14</x:v>
+      </x:c>
+      <x:c r="B38" s="35" t="n">
+        <x:v>46288</x:v>
+      </x:c>
+      <x:c r="C38" s="34" t="str">
+        <x:v>环境变更</x:v>
+      </x:c>
+      <x:c r="D38" s="34" t="str">
+        <x:v>Mac Studio 本机从 V3.12 快进到 V3.14 并重新部署：新增备份目录绑定挂载 /backups 与 backupdir-init 权限初始化服务、web 镜像内置 postgresql-client、.env 补充 BACKUP_PASSPHRASE / BACKUP_TARGET_DIR 校验</x:v>
+      </x:c>
+      <x:c r="E38" s="34" t="str">
+        <x:v>2d6da6f（本次部署）</x:v>
+      </x:c>
+      <x:c r="F38" s="36" t="str">
+        <x:v>docker compose up --build -d --wait 全部 healthy；/api/health/ready=200、登录页=200；容器内 /backups 属主 qnexus 可写；后台「立即执行手动备份」成功（96.5 MB，backup-2026-09-23T05-47-15-217Z-manual.bin），「验证备份」返回「验证通过：数据库转储与上传文件均可解密读取」，审计记录 backup.start/backup.success</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
style: separate login heading lines (V3.15)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Red1dbadfe72846b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rc1dc9b6b94eb42b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R9ef434d6c1b14e42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R17be6aaaeea34490"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rd4bc2a82e1094b21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rabb3579ccdbc4b7d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1138,6 +1138,26 @@
         <x:v>备份模块测试、后台 E2E、Compose 配置契约与真实容器备份—隔离恢复闭环通过</x:v>
       </x:c>
     </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>V3.15</x:v>
+      </x:c>
+      <x:c r="B38" s="3" t="n">
+        <x:v>46288</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>登录页标题两行增加随字号收敛的 6–10px 间距，避免「欢迎来到」中“来”的竖笔与下一行「品集｜Q Nexus」的分隔线视觉粘连；其余布局、文案与交互保持不变，并增加标题行间距回归检查</x:v>
+      </x:c>
+      <x:c r="E38" t="str">
+        <x:v>本次提交，标签 v3.15</x:v>
+      </x:c>
+      <x:c r="F38" t="str">
+        <x:v>标题行边界回归由 0px 转为约 8px；UI E2E 4 场景、typecheck、lint、build 通过（lint 保留 6 条既有警告，build 保留 3 条既有文件追踪警告）</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
merge: preserve V3.14 deployment record
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R6878acca95d042ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R89e757ffd77b494a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rdc410a4718484287"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rdae203919aa74e55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rb4fd6a8305b54f3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R66cf1b5786034e8d"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat: add backup download and restore drill controls (V3.16)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rdae203919aa74e55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rb4fd6a8305b54f3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R66cf1b5786034e8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R9001bcc0488a4fb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R171df2561aae4352"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rf4c4c9f497224cbf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1179,6 +1179,26 @@
         <x:v>标题行边界回归由 0px 转为约 8px；UI E2E 4 场景、typecheck、lint、build 通过（lint 保留 6 条既有警告，build 保留 3 条既有文件追踪警告）</x:v>
       </x:c>
     </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="str">
+        <x:v>V3.16</x:v>
+      </x:c>
+      <x:c r="B40" s="3" t="n">
+        <x:v>46289</x:v>
+      </x:c>
+      <x:c r="C40" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D40" t="str">
+        <x:v>备份管理页为成功记录增加加密包下载链接与恢复演练按钮；下载再次校验管理员身份并返回对应文件；恢复演练在隔离 PostgreSQL 数据库中核对账号、文章、书目、模板和上传文件，完成后自动清理，不覆盖生产数据库</x:v>
+      </x:c>
+      <x:c r="E40" t="str">
+        <x:v>标签 v3.16</x:v>
+      </x:c>
+      <x:c r="F40" t="str">
+        <x:v>备份模块测试、后台页面 E2E、真实 Compose 中的文件下载与隔离恢复演练通过</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1647,6 +1667,34 @@
         <x:v>fix: 完整备份与隔离数据库恢复演练</x:v>
       </x:c>
     </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>V3.15</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>e70b3b5</x:v>
+      </x:c>
+      <x:c r="C35" s="3" t="n">
+        <x:v>46288</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>style: 登录页标题两行增加自适应间距</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>V3.16</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>v3.16</x:v>
+      </x:c>
+      <x:c r="C36" s="3" t="n">
+        <x:v>46289</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>feat: 后台下载备份并执行隔离恢复演练</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record the local deployment to V3.16
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R9001bcc0488a4fb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R171df2561aae4352"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rf4c4c9f497224cbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R01107432e2624e38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R11519c22c4284646"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Ra310c0fc1d7b464b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1180,23 +1180,43 @@
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" t="str">
+      <x:c r="A40" s="26" t="str">
         <x:v>V3.16</x:v>
       </x:c>
-      <x:c r="B40" s="3" t="n">
+      <x:c r="B40" s="43" t="n">
         <x:v>46289</x:v>
       </x:c>
-      <x:c r="C40" t="str">
-        <x:v>小型修改</x:v>
-      </x:c>
-      <x:c r="D40" t="str">
+      <x:c r="C40" s="27" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D40" s="27" t="str">
         <x:v>备份管理页为成功记录增加加密包下载链接与恢复演练按钮；下载再次校验管理员身份并返回对应文件；恢复演练在隔离 PostgreSQL 数据库中核对账号、文章、书目、模板和上传文件，完成后自动清理，不覆盖生产数据库</x:v>
       </x:c>
-      <x:c r="E40" t="str">
+      <x:c r="E40" s="27" t="str">
         <x:v>标签 v3.16</x:v>
       </x:c>
-      <x:c r="F40" t="str">
+      <x:c r="F40" s="28" t="str">
         <x:v>备份模块测试、后台页面 E2E、真实 Compose 中的文件下载与隔离恢复演练通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="33" t="str">
+        <x:v>V3.16</x:v>
+      </x:c>
+      <x:c r="B41" s="35" t="n">
+        <x:v>46289</x:v>
+      </x:c>
+      <x:c r="C41" s="34" t="str">
+        <x:v>环境变更</x:v>
+      </x:c>
+      <x:c r="D41" s="34" t="str">
+        <x:v>Mac Studio 本机从 V3.14 快进到 V3.16 并重新部署：V3.15 登录标题分行、V3.16 后台备份支持下载与隔离恢复演练（无迁移、无 compose 变更）</x:v>
+      </x:c>
+      <x:c r="E41" s="34" t="str">
+        <x:v>184145c（本次部署）</x:v>
+      </x:c>
+      <x:c r="F41" s="36" t="str">
+        <x:v>docker compose up --build -d --wait 全部 healthy；/api/health/ready=200、登录页=200；后台备份文件下载成功；隔离恢复演练通过（审计 backup.restore_drill.success：账号 16、文章 24、书目 5、模板 3、上传文件 34，生产库未改动）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix: unify Asia/Shanghai date display and aggregate template downloads across versions (V3.17)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R01107432e2624e38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R11519c22c4284646"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Ra310c0fc1d7b464b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R926699bf71254cd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R2fb972cad0a943eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R42659481e2644293"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1200,23 +1200,43 @@
       </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="33" t="str">
+      <x:c r="A41" s="29" t="str">
         <x:v>V3.16</x:v>
       </x:c>
-      <x:c r="B41" s="35" t="n">
+      <x:c r="B41" s="31" t="n">
         <x:v>46289</x:v>
       </x:c>
-      <x:c r="C41" s="34" t="str">
+      <x:c r="C41" s="30" t="str">
         <x:v>环境变更</x:v>
       </x:c>
-      <x:c r="D41" s="34" t="str">
+      <x:c r="D41" s="30" t="str">
         <x:v>Mac Studio 本机从 V3.14 快进到 V3.16 并重新部署：V3.15 登录标题分行、V3.16 后台备份支持下载与隔离恢复演练（无迁移、无 compose 变更）</x:v>
       </x:c>
-      <x:c r="E41" s="34" t="str">
+      <x:c r="E41" s="30" t="str">
         <x:v>184145c（本次部署）</x:v>
       </x:c>
-      <x:c r="F41" s="36" t="str">
+      <x:c r="F41" s="30" t="str">
         <x:v>docker compose up --build -d --wait 全部 healthy；/api/health/ready=200、登录页=200；后台备份文件下载成功；隔离恢复演练通过（审计 backup.restore_drill.success：账号 16、文章 24、书目 5、模板 3、上传文件 34，生产库未改动）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="33" t="str">
+        <x:v>V3.17</x:v>
+      </x:c>
+      <x:c r="B42" s="35" t="n">
+        <x:v>46289</x:v>
+      </x:c>
+      <x:c r="C42" s="34" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D42" s="34" t="str">
+        <x:v>修复两处统计显示缺陷（用户反馈）：① 全站日期时间比实际少 8 小时（备份列表 02:40 实为 10:40）——容器时区为 UTC，而 12 处页面各自 new Intl.DateTimeFormat("zh-CN", …) 都没带 timeZone；新增共享模块 src/modules/shared/date-format.ts 统一按 Asia/Shanghai 渲染，并把备份、审计、内容反馈、版本历史、收藏、搜索、文章管理、统计、回收站、首页最近更新等全部切换过去，另加源码守卫用例防止新页面再漏；② 模板下载次数在发布新版本后归零——后台看板与模板详情页只读 active 版本的 download_count，改为按模板汇总所有版本（下载人数按全部版本的下载事件去重）</x:v>
+      </x:c>
+      <x:c r="E42" s="34" t="str">
+        <x:v>本次提交，标签 v3.17</x:v>
+      </x:c>
+      <x:c r="F42" s="34" t="str">
+        <x:v>新增单元用例：格式化器固定上海时区（含跨日边界）、源码守卫（不允许再出现不带 timeZone 的 Intl.DateTimeFormat）、看板跨版本下载汇总、模板详情跨版本下载汇总——四类用例修复前均为红；全量 303 单元用例、12 个 PostgreSQL 容器用例、91 条 e2e 通过；线上实测备份时间显示 10:40、Heat Pipes 下载 3 次·3 人</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1702,17 +1722,31 @@
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" t="str">
+      <x:c r="A36" s="26" t="str">
         <x:v>V3.16</x:v>
       </x:c>
-      <x:c r="B36" t="str">
+      <x:c r="B36" s="27" t="str">
         <x:v>v3.16</x:v>
       </x:c>
-      <x:c r="C36" s="3" t="n">
+      <x:c r="C36" s="43" t="n">
         <x:v>46289</x:v>
       </x:c>
-      <x:c r="D36" t="str">
+      <x:c r="D36" s="28" t="str">
         <x:v>feat: 后台下载备份并执行隔离恢复演练</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="33" t="str">
+        <x:v>V3.17</x:v>
+      </x:c>
+      <x:c r="B37" s="34" t="str">
+        <x:v>（本次提交）</x:v>
+      </x:c>
+      <x:c r="C37" s="35" t="n">
+        <x:v>46289</x:v>
+      </x:c>
+      <x:c r="D37" s="36" t="str">
+        <x:v>fix: 统一上海时区的日期显示 + 模板下载次数按模板汇总所有版本</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix: refresh backup operator and retry Thursday offsite sync (V3.19)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1772,6 +1772,26 @@
         </is>
       </c>
     </row>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="45" ht="100" customHeight="1">
+      <c r="A45" s="33" t="str">
+        <v>V3.19</v>
+      </c>
+      <c r="B45" s="46" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C45" s="34" t="str">
+        <v>小型修改</v>
+      </c>
+      <c r="D45" s="34" t="str">
+        <v>修复旧运维镜像：备份先构建，部署显式构建 backup/bootstrap；周四 13:40 主动离机同步，半小时补拉，失败非零，逐包 SHA-256 校验成功后记录完成。</v>
+      </c>
+      <c r="E45" s="34" t="str">
+        <v>v3.19</v>
+      </c>
+      <c r="F45" s="34" t="str">
+        <v>13 条脚本用例通过；lint/typecheck 通过；新版工具 CLI --drill 真实恢复：16账号、25文章、5书目、3模板、35上传文件；离机同步校验通过。</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1783,7 +1803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2519,6 +2539,20 @@
         <is>
           <t>feat: 新增一条命令完成测试、备份、同步与部署的 SSH 部署脚本</t>
         </is>
+      </c>
+    </row>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="39">
+      <c r="A39" t="str" s="33">
+        <v>V3.19</v>
+      </c>
+      <c r="B39" t="str" s="34">
+        <v>v3.19</v>
+      </c>
+      <c r="C39" s="46" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D39" t="str" s="36">
+        <v>fix: 刷新运维镜像及周四离机同步补拉</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: keep V3.19 change log cells readable
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -148,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -240,6 +240,15 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="3" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
+    <xf xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="164" fontId="3" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
+    <xf xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="3" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -1773,22 +1782,22 @@
       </c>
     </row>
     <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="45" ht="100" customHeight="1">
-      <c r="A45" s="33" t="str">
+      <c r="A45" s="49" t="str">
         <v>V3.19</v>
       </c>
-      <c r="B45" s="46" t="n">
+      <c r="B45" s="50" t="n">
         <v>46311</v>
       </c>
-      <c r="C45" s="34" t="str">
+      <c r="C45" s="51" t="str">
         <v>小型修改</v>
       </c>
-      <c r="D45" s="34" t="str">
+      <c r="D45" s="51" t="str">
         <v>修复旧运维镜像：备份先构建，部署显式构建 backup/bootstrap；周四 13:40 主动离机同步，半小时补拉，失败非零，逐包 SHA-256 校验成功后记录完成。</v>
       </c>
-      <c r="E45" s="34" t="str">
+      <c r="E45" s="51" t="str">
         <v>v3.19</v>
       </c>
-      <c r="F45" s="34" t="str">
+      <c r="F45" s="51" t="str">
         <v>13 条脚本用例通过；lint/typecheck 通过；新版工具 CLI --drill 真实恢复：16账号、25文章、5书目、3模板、35上传文件；离机同步校验通过。</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: protect article reading with identity watermarks and private images (V4.0)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1801,6 +1801,26 @@
         <v>13 条脚本用例通过；lint/typecheck 通过；新版工具 CLI --drill 真实恢复：16账号、25文章、5书目、3模板、35上传文件；离机同步校验通过。</v>
       </c>
     </row>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="46" ht="110" customHeight="1">
+      <c r="A46" s="49" t="str">
+        <v>V4.0</v>
+      </c>
+      <c r="B46" s="50" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C46" s="51" t="str">
+        <v>Superpower 需求</v>
+      </c>
+      <c r="D46" s="51" t="str">
+        <v>文章阅读统一显示天脉品集身份水印；读者限制复制、剪切、右键、拖拽及打印；原图登录与内容引用授权；导出审计。编辑预览、搜索反馈和模板下载保持正常。</v>
+      </c>
+      <c r="E46" s="51" t="str">
+        <v>v4.0</v>
+      </c>
+      <c r="F46" s="51" t="str">
+        <v>新增水印/复制/打印/手机明暗主题浏览器验收；图片权限、快照、原图缓存和导出审计回归。完整测试、构建、部署证据见 docs/operations/releases/v4.0.md。</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1812,7 +1832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2562,6 +2582,20 @@
       </c>
       <c r="D39" t="str" s="36">
         <v>fix: 刷新运维镜像及周四离机同步补拉</v>
+      </c>
+    </row>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="40">
+      <c r="A40" t="str" s="33">
+        <v>V4.0</v>
+      </c>
+      <c r="B40" t="str" s="34">
+        <v>v4.0</v>
+      </c>
+      <c r="C40" s="46" t="n">
+        <v>46314</v>
+      </c>
+      <c r="D40" t="str" s="36">
+        <v>feat: article identity watermarks, reader restrictions and private image/export access</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: protect all reading roles and watermark delivered image pixels
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1821,6 +1821,26 @@
         <v>新增水印/复制/打印/手机明暗主题浏览器验收；图片权限、快照、原图缓存和导出审计回归。完整测试、构建、部署证据见 docs/operations/releases/v4.0.md。</v>
       </c>
     </row>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="47" ht="110" customHeight="1">
+      <c r="A47" s="49" t="str">
+        <v>V4.1</v>
+      </c>
+      <c r="B47" s="50" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C47" s="51" t="str">
+        <v>小型修改</v>
+      </c>
+      <c r="D47" s="51" t="str">
+        <v>修复前台复制与图片另存无水印：所有角色前台统一限制复制、右键、拖拽及打印。服务器把账号身份水印合成到图片像素，保存仍带水印。后台编辑和原始存储不变。</v>
+      </c>
+      <c r="E47" s="51" t="str">
+        <v>v4.1</v>
+      </c>
+      <c r="F47" s="51" t="str">
+        <v>三种角色在文章与主题页真实快捷键复制回归通过，图片像素、格式尺寸与身份隔离通过。完整测试、生产构建与部署验收见 docs/operations/releases/v4.1.md。</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1832,7 +1852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2596,6 +2616,20 @@
       </c>
       <c r="D40" t="str" s="36">
         <v>feat: article identity watermarks, reader restrictions and private image/export access</v>
+      </c>
+    </row>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="41">
+      <c r="A41" t="str" s="33">
+        <v>V4.1</v>
+      </c>
+      <c r="B41" t="str" s="34">
+        <v>v4.1</v>
+      </c>
+      <c r="C41" s="46" t="n">
+        <v>46314</v>
+      </c>
+      <c r="D41" t="str" s="36">
+        <v>fix: protect all reading roles and embed identity watermarks in image pixels</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: bypass legacy public image cache in protected reading
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -1832,7 +1832,7 @@
         <v>小型修改</v>
       </c>
       <c r="D47" s="51" t="str">
-        <v>修复前台复制与图片另存无水印：所有角色前台统一限制复制、右键、拖拽及打印。服务器把账号身份水印合成到图片像素，保存仍带水印。后台编辑和原始存储不变。</v>
+        <v>修复前台复制与图片另存无水印：所有角色前台统一限制复制、右键、拖拽及打印。服务器把账号身份水印合成到图片像素，保存仍带水印。更新图片地址绕过旧公开缓存。后台编辑和原始存储不变。</v>
       </c>
       <c r="E47" s="51" t="str">
         <v>v4.1</v>
@@ -2619,16 +2619,16 @@
       </c>
     </row>
     <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="41">
-      <c r="A41" t="str" s="33">
+      <c r="A41" s="33" t="str">
         <v>V4.1</v>
       </c>
-      <c r="B41" t="str" s="34">
+      <c r="B41" s="34" t="str">
         <v>v4.1</v>
       </c>
       <c r="C41" s="46" t="n">
         <v>46314</v>
       </c>
-      <c r="D41" t="str" s="36">
+      <c r="D41" s="36" t="str">
         <v>fix: protect all reading roles and embed identity watermarks in image pixels</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: place article watermark beneath text and soften image underprint
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1841,6 +1841,26 @@
         <v>三种角色在文章与主题页真实快捷键复制回归通过，图片像素、格式尺寸与身份隔离通过。完整测试、生产构建与部署验收见 docs/operations/releases/v4.1.md。</v>
       </c>
     </row>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="48" ht="110" customHeight="1">
+      <c r="A48" s="49" t="str">
+        <v>V4.2</v>
+      </c>
+      <c r="B48" s="50" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C48" s="51" t="str">
+        <v>小型修改</v>
+      </c>
+      <c r="D48" s="51" t="str">
+        <v>阅读水印调整：文章水印放到正文下方并调淡。图片使用更浅的底纹与 darken 混合，避免盖浅深色文字。保存后的身份水印和复制、打印限制继续有效。</v>
+      </c>
+      <c r="E48" s="51" t="str">
+        <v>v4.2</v>
+      </c>
+      <c r="F48" s="51" t="str">
+        <v>深色文字像素与底纹层级回归、原有图片访问及真实复制检查通过。实际图片及手机明暗主题查看，构建和部署验收见 docs/operations/releases/v4.2.md。</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1852,7 +1872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2630,6 +2650,20 @@
       </c>
       <c r="D41" s="36" t="str">
         <v>fix: protect all reading roles and embed identity watermarks in image pixels</v>
+      </c>
+    </row>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="42">
+      <c r="A42" t="str" s="33">
+        <v>V4.2</v>
+      </c>
+      <c r="B42" t="str" s="34">
+        <v>v4.2</v>
+      </c>
+      <c r="C42" s="46" t="n">
+        <v>46314</v>
+      </c>
+      <c r="D42" t="str" s="36">
+        <v>fix: render watermarks beneath article text and preserve dark image ink</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: unify reading and atomic content workflows in V5.0
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R09f1b43ea4f14581"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R8045e0c2838040d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Re698468177e84a76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R8c5f5248e3564c20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rfe240d246fbb4df1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R0fe0ddf824f94d92"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -150,7 +150,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="53">
+  <x:cellXfs count="59">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0"/>
@@ -253,6 +253,24 @@
     </x:xf>
     <x:xf numFmtId="164" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1883,6 +1901,46 @@
         <x:v>大尺寸图片红绿回归及原图保留、像素上限测试通过。全站图片与生产部署验收见 docs/operations/releases/v4.3.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="50" ht="105" customHeight="1">
+      <x:c r="A50" s="53" t="str">
+        <x:v>V4.4</x:v>
+      </x:c>
+      <x:c r="B50" s="52" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="C50" s="54" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D50" s="54" t="str">
+        <x:v>补记已交付的栏目与主题排序修复：前后台顺序一致、同级排序原子归一、新建追加末尾。</x:v>
+      </x:c>
+      <x:c r="E50" s="54" t="str">
+        <x:v>v4.4</x:v>
+      </x:c>
+      <x:c r="F50" s="54" t="str">
+        <x:v>依据现有 Git 标签与 docs/operations/releases/v4.4.md 补记；本次不重复修改或部署 V4.4。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="160" customHeight="1">
+      <x:c r="A51" s="53" t="str">
+        <x:v>V5.0</x:v>
+      </x:c>
+      <x:c r="B51" s="52" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="C51" s="54" t="str">
+        <x:v>Superpower 需求</x:v>
+      </x:c>
+      <x:c r="D51" s="54" t="str">
+        <x:v>架构巡检四项修复：统一已发布文章阅读；编辑占用与版本校验；生命周期与审计原子提交；后台和 CLI 共用恢复演练。</x:v>
+      </x:c>
+      <x:c r="E51" s="54" t="str">
+        <x:v>v5.0</x:v>
+      </x:c>
+      <x:c r="F51" s="54" t="str">
+        <x:v>全量本地 363 项、真实 PostgreSQL 18 项通过；真实自动保存、接管拒写与同账号冲突回归通过。完整浏览器、构建、容器恢复及生产部署验收见 docs/operations/releases/v5.0.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2697,6 +2755,34 @@
         <x:v>验收见 docs/operations/releases/v4.3.md；Git 标签定位关联提交。</x:v>
       </x:c>
     </x:row>
+    <x:row r="44" ht="70" customHeight="1">
+      <x:c r="A44" s="55" t="str">
+        <x:v>V4.4</x:v>
+      </x:c>
+      <x:c r="B44" s="56" t="str">
+        <x:v>v4.4</x:v>
+      </x:c>
+      <x:c r="C44" s="57" t="str">
+        <x:v>补记既有排序版本</x:v>
+      </x:c>
+      <x:c r="D44" s="58" t="str">
+        <x:v>运行提交 fd0034b；验收见 docs/operations/releases/v4.4.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="70" customHeight="1">
+      <x:c r="A45" s="55" t="str">
+        <x:v>V5.0</x:v>
+      </x:c>
+      <x:c r="B45" s="56" t="str">
+        <x:v>v5.0</x:v>
+      </x:c>
+      <x:c r="C45" s="57" t="str">
+        <x:v>2026-10-20 架构一致性修复</x:v>
+      </x:c>
+      <x:c r="D45" s="58" t="str">
+        <x:v>Git 标签 v5.0 定位交付提交；验收见 docs/operations/releases/v5.0.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat: add administrator learning participation statistics (V6.0)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R8c5f5248e3564c20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rfe240d246fbb4df1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R0fe0ddf824f94d92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R2587248b00b64922"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Ra61274bb42264e10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Re93a5929bf434830"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1941,6 +1941,26 @@
         <x:v>全量本地 363 项、真实 PostgreSQL 18 项通过；真实自动保存、接管拒写与同账号冲突回归通过。完整浏览器、构建、容器恢复及生产部署验收见 docs/operations/releases/v5.0.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="52" ht="165" customHeight="1">
+      <x:c r="A52" s="53" t="str">
+        <x:v>V6.0</x:v>
+      </x:c>
+      <x:c r="B52" s="52" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="C52" s="54" t="str">
+        <x:v>Superpower 需求</x:v>
+      </x:c>
+      <x:c r="D52" s="54" t="str">
+        <x:v>管理员学习参与统计：总览、人员、内容三视图；实名阅读、模板下载与登录明细；有效阅读与活跃时长，收藏数量、汇总Excel审计、两年保留；恢复账号和测试账号排除。无登录说明弹窗。</x:v>
+      </x:c>
+      <x:c r="E52" s="54" t="str">
+        <x:v>v6.0</x:v>
+      </x:c>
+      <x:c r="F52" s="54" t="str">
+        <x:v>采集阈值、并发去重、跨日、权限与历史未采集红绿回归；全量本地、真实PostgreSQL、浏览器、构建及生产部署验收见 docs/operations/releases/v6.0.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2783,6 +2803,20 @@
         <x:v>Git 标签 v5.0 定位交付提交；验收见 docs/operations/releases/v5.0.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="46" ht="70" customHeight="1">
+      <x:c r="A46" s="55" t="str">
+        <x:v>V6.0</x:v>
+      </x:c>
+      <x:c r="B46" s="56" t="str">
+        <x:v>v6.0</x:v>
+      </x:c>
+      <x:c r="C46" s="57" t="str">
+        <x:v>2026-10-21 管理员学习参与统计</x:v>
+      </x:c>
+      <x:c r="D46" s="58" t="str">
+        <x:v>Git标签 v6.0 定位交付提交；验收见 docs/operations/releases/v6.0.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
refactor: deepen reading, reports and draft sessions (V7.0)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R2587248b00b64922"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Ra61274bb42264e10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Re93a5929bf434830"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R5e5c487fddd64ef3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R65396f797dcb48ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R8bbf0d8ac5fc474e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1961,6 +1961,26 @@
         <x:v>采集阈值、并发去重、跨日、权限与历史未采集红绿回归；全量本地、真实PostgreSQL、浏览器、构建及生产部署验收见 docs/operations/releases/v6.0.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="53" ht="165" customHeight="1">
+      <x:c r="A53" s="53" t="str">
+        <x:v>V7.0</x:v>
+      </x:c>
+      <x:c r="B53" s="52" t="d">
+        <x:v>2026-10-22T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C53" s="54" t="str">
+        <x:v>Superpower 需求</x:v>
+      </x:c>
+      <x:c r="D53" s="54" t="str">
+        <x:v>架构深化三项：阅读时序独立 module；人员导出专用汇总、统计分组索引及独立知识缺口查询；编辑草稿统一自动保存、离线恢复与冲突时序，保护在途输入和恢复副本。</x:v>
+      </x:c>
+      <x:c r="E53" s="54" t="str">
+        <x:v>v7.0</x:v>
+      </x:c>
+      <x:c r="F53" s="54" t="str">
+        <x:v>阅读与草稿交错时序红绿回归；人员专用汇总、独立知识缺口读取、全量验证及部署验收见 docs/operations/releases/v7.0.md（验收进行中）。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2817,6 +2837,20 @@
         <x:v>Git标签 v6.0 定位交付提交；验收见 docs/operations/releases/v6.0.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="47" ht="70" customHeight="1">
+      <x:c r="A47" s="55" t="str">
+        <x:v>V7.0</x:v>
+      </x:c>
+      <x:c r="B47" s="56" t="str">
+        <x:v>v7.0</x:v>
+      </x:c>
+      <x:c r="C47" s="57" t="str">
+        <x:v>2026-10-22 架构深化三项</x:v>
+      </x:c>
+      <x:c r="D47" s="58" t="str">
+        <x:v>Git标签 v7.0 定位交付提交；验收见 docs/operations/releases/v7.0.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record V7.0 production and container acceptance
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R5e5c487fddd64ef3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R65396f797dcb48ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R8bbf0d8ac5fc474e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R3176266722c8447f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R0d668df2959145f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R9e1d434d89884cb4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1978,7 +1978,7 @@
         <x:v>v7.0</x:v>
       </x:c>
       <x:c r="F53" s="54" t="str">
-        <x:v>阅读与草稿交错时序红绿回归；人员专用汇总、独立知识缺口读取、全量验证及部署验收见 docs/operations/releases/v7.0.md（验收进行中）。</x:v>
+        <x:v>全量本地409项、真实PostgreSQL19项、完整浏览器102项与新增离线恢复回归通过；生产镜像隔离容器运行、备份恢复及quality-server升级验收通过。详见 docs/operations/releases/v7.0.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(admin): adopt structured console UI (V8.0)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R3176266722c8447f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R0d668df2959145f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R9e1d434d89884cb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R584277bb52f54b3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R7ddc6a98587d4e68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R9210259f690b4345"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1981,6 +1981,26 @@
         <x:v>全量本地409项、真实PostgreSQL19项、完整浏览器102项与新增离线恢复回归通过；生产镜像隔离容器运行、备份恢复及quality-server升级验收通过。详见 docs/operations/releases/v7.0.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="54" ht="165" customHeight="1">
+      <x:c r="A54" s="53" t="str">
+        <x:v>V8.0</x:v>
+      </x:c>
+      <x:c r="B54" s="52" t="d">
+        <x:v>2026-10-22T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C54" s="54" t="str">
+        <x:v>Superpower 需求</x:v>
+      </x:c>
+      <x:c r="D54" s="54" t="str">
+        <x:v>后台结构化控制台：统一分组侧栏、紧凑排版与按钮层级；账号筛选分页和按需弹窗；文章表格与按需归档；学习统计指标和人员摘要优先展示，保留权限及统计口径。</x:v>
+      </x:c>
+      <x:c r="E54" s="54" t="str">
+        <x:v>v8.0</x:v>
+      </x:c>
+      <x:c r="F54" s="54" t="str">
+        <x:v>本地与部署验收记录见 docs/operations/releases/v8.0.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2851,6 +2871,20 @@
         <x:v>Git标签 v7.0 定位交付提交；验收见 docs/operations/releases/v7.0.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="48" ht="70" customHeight="1">
+      <x:c r="A48" s="55" t="str">
+        <x:v>V8.0</x:v>
+      </x:c>
+      <x:c r="B48" s="56" t="str">
+        <x:v>v8.0</x:v>
+      </x:c>
+      <x:c r="C48" s="57" t="str">
+        <x:v>2026-10-22 后台结构化控制台</x:v>
+      </x:c>
+      <x:c r="D48" s="58" t="str">
+        <x:v>Git 标签 v8.0 定位交付提交；设计和验收见 design-qa.md、docs/operations/releases/v8.0.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(release): record V8.0 deployment acceptance
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R584277bb52f54b3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R7ddc6a98587d4e68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R9210259f690b4345"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R9365e2dda104478a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Re1adfed13bac4efd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rc1feaae70f034e0c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1998,7 +1998,7 @@
         <x:v>v8.0</x:v>
       </x:c>
       <x:c r="F54" s="54" t="str">
-        <x:v>本地与部署验收记录见 docs/operations/releases/v8.0.md。</x:v>
+        <x:v>本地409项、真实PostgreSQL19项；浏览器104项覆盖（90项通过及14项修正/隔离复测通过）；构建、视觉对照、390px和深色验证通过。quality-server升级V8.0，备份成功、服务healthy，105账号/26文章/9模板/347版本与升级前一致；详见 docs/operations/releases/v8.0.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs(release): record V9.0 reading design and local acceptance
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R9365e2dda104478a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Re1adfed13bac4efd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rc1feaae70f034e0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R032ee8a92152487d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R281f3c4e92dc4a91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rde364471396447d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2001,6 +2001,26 @@
         <x:v>本地409项、真实PostgreSQL19项；浏览器104项覆盖（90项通过及14项修正/隔离复测通过）；构建、视觉对照、390px和深色验证通过。quality-server升级V8.0，备份成功、服务healthy，105账号/26文章/9模板/347版本与升级前一致；详见 docs/operations/releases/v8.0.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="55" ht="165" customHeight="1">
+      <x:c r="A55" s="53" t="str">
+        <x:v>V9.0</x:v>
+      </x:c>
+      <x:c r="B55" s="52" t="d">
+        <x:v>2026-10-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C55" s="54" t="str">
+        <x:v>Superpower 需求</x:v>
+      </x:c>
+      <x:c r="D55" s="54" t="str">
+        <x:v>文章阅读模板首批：限域浅深色Tokens、真实知识树和目录、元信息重排、手机单栏；修复公式排版及Mermaid内容/主题更新，提高浅色Warning标题对比度，保留内容保护和原业务入口。</x:v>
+      </x:c>
+      <x:c r="E55" s="54" t="str">
+        <x:v>e9553fc–4d9bc34（本地；v9.0待发布）</x:v>
+      </x:c>
+      <x:c r="F55" s="54" t="str">
+        <x:v>本地验收见 docs/design/editorial-reading-v9.0/acceptance.md；部署和GitHub/tag发布待用户批准，未记为生产验收通过。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2885,6 +2905,20 @@
         <x:v>Git 标签 v8.0 定位交付提交；设计和验收见 design-qa.md、docs/operations/releases/v8.0.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="49" ht="70" customHeight="1">
+      <x:c r="A49" s="55" t="str">
+        <x:v>V9.0</x:v>
+      </x:c>
+      <x:c r="B49" s="56" t="str">
+        <x:v>e9553fc–4d9bc34；v9.0待发布</x:v>
+      </x:c>
+      <x:c r="C49" s="57" t="str">
+        <x:v>2026-10-28 文章阅读模板首批</x:v>
+      </x:c>
+      <x:c r="D49" s="58" t="str">
+        <x:v>本地验收见 docs/operations/releases/v9.0.md；部署后补充运行SHA与验收，再发布GitHub及标签。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(release): record V9.0 deployment acceptance
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R032ee8a92152487d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R281f3c4e92dc4a91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rde364471396447d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rd849f55d65b04e8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R8fc8e327d6df4551"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R43aba8e3ed6d45f1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2015,10 +2015,10 @@
         <x:v>文章阅读模板首批：限域浅深色Tokens、真实知识树和目录、元信息重排、手机单栏；修复公式排版及Mermaid内容/主题更新，提高浅色Warning标题对比度，保留内容保护和原业务入口。</x:v>
       </x:c>
       <x:c r="E55" s="54" t="str">
-        <x:v>e9553fc–4d9bc34（本地；v9.0待发布）</x:v>
+        <x:v>e9553fc–4d9bc34；运行c7763b3；v9.0定位最终验收记录</x:v>
       </x:c>
       <x:c r="F55" s="54" t="str">
-        <x:v>本地验收见 docs/design/editorial-reading-v9.0/acceptance.md；部署和GitHub/tag发布待用户批准，未记为生产验收通过。</x:v>
+        <x:v>2026-10-28 quality-server部署V9.0；加密备份34fd5306校验55条目通过；服务healthy，105账号/26文章/14模板/347版本保持；登录页、新版CSS及未登录访问保护通过。连接器无法访问LAN，未做已登录生产交互；详见docs/operations/releases/v9.0.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2910,13 +2910,13 @@
         <x:v>V9.0</x:v>
       </x:c>
       <x:c r="B49" s="56" t="str">
-        <x:v>e9553fc–4d9bc34；v9.0待发布</x:v>
+        <x:v>v9.0</x:v>
       </x:c>
       <x:c r="C49" s="57" t="str">
         <x:v>2026-10-28 文章阅读模板首批</x:v>
       </x:c>
       <x:c r="D49" s="58" t="str">
-        <x:v>本地验收见 docs/operations/releases/v9.0.md；部署后补充运行SHA与验收，再发布GitHub及标签。</x:v>
+        <x:v>运行应用源码c7763b3；部署验收及最终GitHub/tag记录见docs/operations/releases/v9.0.md；最终记录提交同步部署机后再发布。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(ui): complete editorial design across Q-Nexus V10.0
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rd849f55d65b04e8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R8fc8e327d6df4551"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R43aba8e3ed6d45f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R9504c0fc40fa4c0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rab8cf70a869a4646"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R1af49c1fffa24350"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2021,6 +2021,26 @@
         <x:v>2026-10-28 quality-server部署V9.0；加密备份34fd5306校验55条目通过；服务healthy，105账号/26文章/14模板/347版本保持；登录页、新版CSS及未登录访问保护通过。连接器无法访问LAN，未做已登录生产交互；详见docs/operations/releases/v9.0.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="56" ht="180" customHeight="1">
+      <x:c r="A56" s="53" t="str">
+        <x:v>V10.0</x:v>
+      </x:c>
+      <x:c r="B56" s="52" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C56" s="54" t="str">
+        <x:v>Superpower 需求</x:v>
+      </x:c>
+      <x:c r="D56" s="54" t="str">
+        <x:v>完整实施现代编辑型UI：首页专题/真实搜索/知识分类/最近更新与新人入口；品质及散热内联全文、独立目录锚点；新人路线/书单/模板/搜索/收藏与登录、后台统一浅深色；修复主题搜索归属、浮层关闭与请求竞态。</x:v>
+      </x:c>
+      <x:c r="E56" s="54" t="str">
+        <x:v>v10.0</x:v>
+      </x:c>
+      <x:c r="F56" s="54" t="str">
+        <x:v>本地70文件417项、真实PostgreSQL19项通过；全套浏览器122项通过，失败路径修复后专项复验通过；阅读14项及分类/保护/全站28项通过。构建、格式、类型、lint与Compose通过。Ego桌面/手机浅深及主要入口视觉通过；部署验收待完成，见docs/operations/releases/v10.0.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2919,6 +2939,20 @@
         <x:v>运行应用源码c7763b3；部署验收及最终GitHub/tag记录见docs/operations/releases/v9.0.md；最终记录提交同步部署机后再发布。</x:v>
       </x:c>
     </x:row>
+    <x:row r="50" ht="70" customHeight="1">
+      <x:c r="A50" s="55" t="str">
+        <x:v>V10.0</x:v>
+      </x:c>
+      <x:c r="B50" s="56" t="str">
+        <x:v>v10.0</x:v>
+      </x:c>
+      <x:c r="C50" s="57" t="str">
+        <x:v>2026-10-29 完整现代编辑型UI</x:v>
+      </x:c>
+      <x:c r="D50" s="58" t="str">
+        <x:v>Git标签v10.0定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.0.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(release): record V10.0 visual and LAN acceptance
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R9504c0fc40fa4c0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rab8cf70a869a4646"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R1af49c1fffa24350"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R665ac46f8128483e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R12e6ff6a3c8c4001"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R9da03381bf4a4b7b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2032,13 +2032,13 @@
         <x:v>Superpower 需求</x:v>
       </x:c>
       <x:c r="D56" s="54" t="str">
-        <x:v>完整实施现代编辑型UI：首页专题/真实搜索/知识分类/最近更新与新人入口；品质及散热内联全文、独立目录锚点；新人路线/书单/模板/搜索/收藏与登录、后台统一浅深色；修复主题搜索归属、浮层关闭与请求竞态。</x:v>
+        <x:v>完整实施现代编辑型UI：首页专题/真实搜索/知识分类/最近更新与新人入口；品质及散热内联全文、独立目录锚点；新人路线/书单/模板/搜索/收藏与登录、后台统一浅深色；修复主题搜索归属、浮层关闭与请求竞态；受保护图片增加服务端诊断。</x:v>
       </x:c>
       <x:c r="E56" s="54" t="str">
         <x:v>v10.0</x:v>
       </x:c>
       <x:c r="F56" s="54" t="str">
-        <x:v>本地70文件417项、真实PostgreSQL19项通过；全套浏览器122项通过，失败路径修复后专项复验通过；阅读14项及分类/保护/全站28项通过。构建、格式、类型、lint与Compose通过。Ego桌面/手机浅深及主要入口视觉通过；部署验收待完成，见docs/operations/releases/v10.0.md。</x:v>
+        <x:v>本地417项、真实PostgreSQL19项通过；业务浏览器122项及失败路径复验通过；分类/保护28项、阅读14项、补充图片7项通过。格式/类型/lint/构建/Compose通过。Ego视觉及生产Lou会话主要入口、浅深/手机验收通过；图片重建恢复并经重启复验。备份a199ab98校验55条目，业务105/26/14/347不变；详见v10.0发布记录。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix(ui): refine recommended books layout V10.1
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R665ac46f8128483e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R12e6ff6a3c8c4001"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R9da03381bf4a4b7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Raf155a8ddf1e4051"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R3f53d9abec56453d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rc257b1a387184b90"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2041,6 +2041,26 @@
         <x:v>本地417项、真实PostgreSQL19项通过；业务浏览器122项及失败路径复验通过；分类/保护28项、阅读14项、补充图片7项通过。格式/类型/lint/构建/Compose通过。Ego视觉及生产Lou会话主要入口、浅深/手机验收通过；图片重建恢复并经重启复验。备份a199ab98校验55条目，业务105/26/14/347不变；详见v10.0发布记录。</x:v>
       </x:c>
     </x:row>
+    <x:row r="57" ht="180" customHeight="1">
+      <x:c r="A57" s="53" t="str">
+        <x:v>V10.1</x:v>
+      </x:c>
+      <x:c r="B57" s="52" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C57" s="54" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D57" s="54" t="str">
+        <x:v>推荐书单改为两列分类卡片，放大完整封面；书名/作者/推荐理由/适合人群分层；顶部真实书目数和分类锚点；适配手机及浅深色。</x:v>
+      </x:c>
+      <x:c r="E57" s="54" t="str">
+        <x:v>v10.1</x:v>
+      </x:c>
+      <x:c r="F57" s="54" t="str">
+        <x:v>书单管理3项、响应式/无障碍2项、格式/类型/lint/构建通过；Ego桌面/手机浅深布局检查通过。生产验收待完成，见docs/operations/releases/v10.1.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2953,6 +2973,20 @@
         <x:v>Git标签v10.0定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.0.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="51" ht="70" customHeight="1">
+      <x:c r="A51" s="55" t="str">
+        <x:v>V10.1</x:v>
+      </x:c>
+      <x:c r="B51" s="56" t="str">
+        <x:v>v10.1</x:v>
+      </x:c>
+      <x:c r="C51" s="57" t="str">
+        <x:v>2026-10-29 推荐书单书架排版</x:v>
+      </x:c>
+      <x:c r="D51" s="58" t="str">
+        <x:v>Git标签v10.1定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.1.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(release): record V10.1 books visual acceptance
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Raf155a8ddf1e4051"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R3f53d9abec56453d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rc257b1a387184b90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R1e37151b63df44d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rd421a1ff04aa425f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rc3080e841fd84fc4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2058,7 +2058,7 @@
         <x:v>v10.1</x:v>
       </x:c>
       <x:c r="F57" s="54" t="str">
-        <x:v>书单管理3项、响应式/无障碍2项、格式/类型/lint/构建通过；Ego桌面/手机浅深布局检查通过。生产验收待完成，见docs/operations/releases/v10.1.md。</x:v>
+        <x:v>书目管理3项、响应式/无障碍2项及格式/类型/lint/构建通过。Ego生产1440浅深、375手机对照及分类跳转通过，5张封面完整显示。备份94570435校验64条目；业务105账号/5书目/5分类/33文章不变。发布验收详见docs/operations/releases/v10.1.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(books): implement selected cover gallery V10.2
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R1e37151b63df44d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rd421a1ff04aa425f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rc3080e841fd84fc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rdebdb5250cc64616"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rb6086e7770fa4155"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R175e88f97c2e45f3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2061,6 +2061,26 @@
         <x:v>书目管理3项、响应式/无障碍2项及格式/类型/lint/构建通过。Ego生产1440浅深、375手机对照及分类跳转通过，5张封面完整显示。备份94570435校验64条目；业务105账号/5书目/5分类/33文章不变。发布验收详见docs/operations/releases/v10.1.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="58" ht="180" customHeight="1">
+      <x:c r="A58" s="53" t="str">
+        <x:v>V10.2</x:v>
+      </x:c>
+      <x:c r="B58" s="52" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C58" s="54" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D58" s="54" t="str">
+        <x:v>按用户选择的第二张封面书墙实施四列大封面画廊，顶部真实分类筛选与选中态，网址/历史恢复及空态；保留真实书目与图片保护，适配浅深色和手机。</x:v>
+      </x:c>
+      <x:c r="E58" s="54" t="str">
+        <x:v>v10.2</x:v>
+      </x:c>
+      <x:c r="F58" s="54" t="str">
+        <x:v>干净隔离浏览器5项通过，含管理、分类筛选/历史/空态、320/375/768/1440浅深布局与严重无障碍；格式/类型/lint/生产构建通过。备份cb6de60d校验65条目；待生产真实封面视觉对照。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2987,6 +3007,20 @@
         <x:v>Git标签v10.1定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.1.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="52" ht="70" customHeight="1">
+      <x:c r="A52" s="55" t="str">
+        <x:v>V10.2</x:v>
+      </x:c>
+      <x:c r="B52" s="56" t="str">
+        <x:v>v10.2</x:v>
+      </x:c>
+      <x:c r="C52" s="57" t="str">
+        <x:v>2026-10-29 已选第二方案封面书墙</x:v>
+      </x:c>
+      <x:c r="D52" s="58" t="str">
+        <x:v>Git标签v10.2定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.2.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(release): accept selected V10.2 cover gallery
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rdebdb5250cc64616"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rb6086e7770fa4155"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R175e88f97c2e45f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R5941f8273fec4225"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rf73f30fe81f0487f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R80b902d15483432a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2078,7 +2078,7 @@
         <x:v>v10.2</x:v>
       </x:c>
       <x:c r="F58" s="54" t="str">
-        <x:v>干净隔离浏览器5项通过，含管理、分类筛选/历史/空态、320/375/768/1440浅深布局与严重无障碍；格式/类型/lint/生产构建通过。备份cb6de60d校验65条目；待生产真实封面视觉对照。</x:v>
+        <x:v>隔离浏览器5项及最终筛选/响应式2项复验通过；格式/lint/类型/生产构建通过。Ego生产5张封面、分类筛选、浅深/375手机/200%文字与选定第二图同尺寸全景及字体局部对照通过，QA passed。备份cb6de60d校验65条目；业务105账号/5书目/5分类/33文章不变。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
chore(books): prepare verified front cover V10.3
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R5941f8273fec4225"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rf73f30fe81f0487f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R80b902d15483432a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R39d5354977144010"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R0061091bb00b4703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R5fe2da493a6f4409"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2081,6 +2081,26 @@
         <x:v>隔离浏览器5项及最终筛选/响应式2项复验通过；格式/lint/类型/生产构建通过。Ego生产5张封面、分类筛选、浅深/375手机/200%文字与选定第二图同尺寸全景及字体局部对照通过，QA passed。备份cb6de60d校验65条目；业务105账号/5书目/5分类/33文章不变。</x:v>
       </x:c>
     </x:row>
+    <x:row r="59" ht="180" customHeight="1">
+      <x:c r="A59" s="53" t="str">
+        <x:v>V10.3</x:v>
+      </x:c>
+      <x:c r="B59" s="52" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C59" s="54" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D59" s="54" t="str">
+        <x:v>从豆瓣阅读核验并取得《质量免费》同款正面封面，替换侧面立体图；原图与来源归档，保留原书目文字及图片授权/身份水印。</x:v>
+      </x:c>
+      <x:c r="E59" s="54" t="str">
+        <x:v>v10.3</x:v>
+      </x:c>
+      <x:c r="F59" s="54" t="str">
+        <x:v>书名/作者/ISBN核验，JPEG330×495可解码，源图SHA256已记录；更换前加密备份6d1cb264，后台替换与视觉验收待完成。见docs/operations/releases/v10.3.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3021,6 +3041,20 @@
         <x:v>Git标签v10.2定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.2.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="53" ht="70" customHeight="1">
+      <x:c r="A53" s="55" t="str">
+        <x:v>V10.3</x:v>
+      </x:c>
+      <x:c r="B53" s="56" t="str">
+        <x:v>v10.3</x:v>
+      </x:c>
+      <x:c r="C53" s="57" t="str">
+        <x:v>2026-10-29 质量免费正面封面</x:v>
+      </x:c>
+      <x:c r="D53" s="58" t="str">
+        <x:v>Git标签v10.3定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.3.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(books): verify front cover replacement V10.3
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R39d5354977144010"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R0061091bb00b4703"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R5fe2da493a6f4409"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R358bebde28ca454f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R0a51dd99466a4d0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R9a116a96c4cf46a6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2098,7 +2098,7 @@
         <x:v>v10.3</x:v>
       </x:c>
       <x:c r="F59" s="54" t="str">
-        <x:v>书名/作者/ISBN核验，JPEG330×495可解码，源图SHA256已记录；更换前加密备份6d1cb264，后台替换与视觉验收待完成。见docs/operations/releases/v10.3.md。</x:v>
+        <x:v>核验豆瓣阅读同款正面封面及ISBN，原图SHA256与受控存储一致。5条书目比较仅目标封面/时间变化；桌面前4封面可见高度均376px，手机375无溢出、5图正常；匿名401、ready200。备份6d1cb264完整性65条目通过，见v10.3记录。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
chore(books): prepare user supplied cover V10.4
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R358bebde28ca454f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R0a51dd99466a4d0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R9a116a96c4cf46a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Ra1d635820f214f91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R859a03623fc94bae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rfb9b73b7a7004712"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2101,6 +2101,26 @@
         <x:v>核验豆瓣阅读同款正面封面及ISBN，原图SHA256与受控存储一致。5条书目比较仅目标封面/时间变化；桌面前4封面可见高度均376px，手机375无溢出、5图正常；匿名401、ready200。备份6d1cb264完整性65条目通过，见v10.3记录。</x:v>
       </x:c>
     </x:row>
+    <x:row r="60" ht="180" customHeight="1">
+      <x:c r="A60" s="53" t="str">
+        <x:v>V10.4</x:v>
+      </x:c>
+      <x:c r="B60" s="52" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C60" s="54" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D60" s="54" t="str">
+        <x:v>按用户指定的1069×1471高清红色漩涡PNG原图维护《质量免费》封面，保留原始分辨率；书名、作者、推荐理由及其他书目不变，沿用图片保护。</x:v>
+      </x:c>
+      <x:c r="E60" s="54" t="str">
+        <x:v>v10.4</x:v>
+      </x:c>
+      <x:c r="F60" s="54" t="str">
+        <x:v>用户指定PNG已核对尺寸1069×1471及SHA256，原样归档。更换前加密备份c93d9dd5，完整性66条目通过；后台上传及桌面/手机验收待完成。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3055,6 +3075,20 @@
         <x:v>Git标签v10.3定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.3.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="54" ht="70" customHeight="1">
+      <x:c r="A54" s="55" t="str">
+        <x:v>V10.4</x:v>
+      </x:c>
+      <x:c r="B54" s="56" t="str">
+        <x:v>v10.4</x:v>
+      </x:c>
+      <x:c r="C54" s="57" t="str">
+        <x:v>2026-10-29 用户指定高清红色漩涡封面</x:v>
+      </x:c>
+      <x:c r="D54" s="58" t="str">
+        <x:v>Git标签v10.4定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.4.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(books): verify user cover replacement V10.4
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Ra1d635820f214f91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R859a03623fc94bae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rfb9b73b7a7004712"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R101d655a5e454057"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rcca4dccfb82a4164"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R7484d87418064ddf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2118,7 +2118,7 @@
         <x:v>v10.4</x:v>
       </x:c>
       <x:c r="F60" s="54" t="str">
-        <x:v>用户指定PNG已核对尺寸1069×1471及SHA256，原样归档。更换前加密备份c93d9dd5，完整性66条目通过；后台上传及桌面/手机验收待完成。</x:v>
+        <x:v>使用用户指定原PNG，1069×1471/1,527,235字节，入库SHA256与源文件一致。仅目标封面/格式/时间变化，其他书目相同；桌面/手机实拍5图正常、无溢出，匿名401、ready200。备份c93d9dd5校验66条目通过；详见v10.4记录。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix: restore protected image rendering and exempt book covers (V10.5)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R101d655a5e454057"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rcca4dccfb82a4164"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R7484d87418064ddf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rbfa535fc8099430a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rff36b7e6770147e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R1989e276ac514426"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2121,6 +2121,26 @@
         <x:v>使用用户指定原PNG，1069×1471/1,527,235字节，入库SHA256与源文件一致。仅目标封面/格式/时间变化，其他书目相同；桌面/手机实拍5图正常、无溢出，匿名401、ready200。备份c93d9dd5校验66条目通过；详见v10.4记录。</x:v>
       </x:c>
     </x:row>
+    <x:row r="61" ht="180" customHeight="1">
+      <x:c r="A61" s="53" t="str">
+        <x:v>V10.5</x:v>
+      </x:c>
+      <x:c r="B61" s="52" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C61" s="54" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D61" s="54" t="str">
+        <x:v>修复Next图片优化器初始化后受控图片500；文章水印改用文字栅格合成，保留SVG限制。书目封面按服务端真实引用返回原图，不再加水印，保留登录鉴权。</x:v>
+      </x:c>
+      <x:c r="E61" s="54" t="str">
+        <x:v>v10.5</x:v>
+      </x:c>
+      <x:c r="F61" s="54" t="str">
+        <x:v>本地418项、PostgreSQL19项、浏览器11项通过，构建/类型/格式/Compose通过。封面原字节校验及Next初始化后文章水印回归通过。备份5d4883b6校验67条目通过。生产验收结果见v10.5发布记录。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3089,6 +3109,20 @@
         <x:v>Git标签v10.4定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.4.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="55" ht="70" customHeight="1">
+      <x:c r="A55" s="55" t="str">
+        <x:v>V10.5</x:v>
+      </x:c>
+      <x:c r="B55" s="56" t="str">
+        <x:v>v10.5</x:v>
+      </x:c>
+      <x:c r="C55" s="57" t="str">
+        <x:v>2026-10-29 修复图片500与封面免水印</x:v>
+      </x:c>
+      <x:c r="D55" s="58" t="str">
+        <x:v>Git标签v10.5定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.5.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record V10.5 deployment acceptance and image checks
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rbfa535fc8099430a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rff36b7e6770147e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R1989e276ac514426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R7bd991603ada4409"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R9f015702649a429e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R26fc0379e42b4e95"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2138,7 +2138,7 @@
         <x:v>v10.5</x:v>
       </x:c>
       <x:c r="F61" s="54" t="str">
-        <x:v>本地418项、PostgreSQL19项、浏览器11项通过，构建/类型/格式/Compose通过。封面原字节校验及Next初始化后文章水印回归通过。备份5d4883b6校验67条目通过。生产验收结果见v10.5发布记录。</x:v>
+        <x:v>本地418项、PostgreSQL19项、浏览器11项通过；字号校正后专项26项及构建再次通过。生产3轮首页优化→5封面→文章图均200，封面SHA逐一匹配原图，文章水印保持；桌面/手机通过。备份67条目校验、数据量不变。提交58529d4/c46cfed；详见v10.5发布记录。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix: simplify inline article metadata and show last publisher (V10.6)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R7bd991603ada4409"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R9f015702649a429e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R26fc0379e42b4e95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rd086c74712274799"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R6e57ce3c1d3a4be5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R4717e819f49c4f35"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2141,6 +2141,26 @@
         <x:v>本地418项、PostgreSQL19项、浏览器11项通过；字号校正后专项26项及构建再次通过。生产3轮首页优化→5封面→文章图均200，封面SHA逐一匹配原图，文章水印保持；桌面/手机通过。备份67条目校验、数据量不变。提交58529d4/c46cfed；详见v10.5发布记录。</x:v>
       </x:c>
     </x:row>
+    <x:row r="62" ht="180" customHeight="1">
+      <x:c r="A62" s="53" t="str">
+        <x:v>V10.6</x:v>
+      </x:c>
+      <x:c r="B62" s="52" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C62" s="54" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D62" s="54" t="str">
+        <x:v>按确认预览统一精简主题文章信息：正文前仅保留更新日期及实际发布操作人，移除重复标题、负责人和阅读页链接。上方标题保留完整阅读入口，目录锚点不丢失。</x:v>
+      </x:c>
+      <x:c r="E62" s="54" t="str">
+        <x:v>v10.6</x:v>
+      </x:c>
+      <x:c r="F62" s="54" t="str">
+        <x:v>本机专项4项、类型/格式通过，Lint无错误。相同源码在隔离环境71文件419项、PostgreSQL19项、浏览器16项通过，生产构建及Compose通过。备份5e1ab24e校验67条目通过。生产逐篇验收结果见v10.6发布记录。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3123,6 +3143,20 @@
         <x:v>Git标签v10.5定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.5.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="56" ht="70" customHeight="1">
+      <x:c r="A56" s="55" t="str">
+        <x:v>V10.6</x:v>
+      </x:c>
+      <x:c r="B56" s="56" t="str">
+        <x:v>v10.6</x:v>
+      </x:c>
+      <x:c r="C56" s="57" t="str">
+        <x:v>2026-10-29 统一精简主题文章重复信息</x:v>
+      </x:c>
+      <x:c r="D56" s="58" t="str">
+        <x:v>Git标签v10.6定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.6.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record V10.6 deployment and per-article acceptance
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rd086c74712274799"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R6e57ce3c1d3a4be5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R4717e819f49c4f35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R97058d8e9cd749e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rf54cd8ca65484898"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R683138d4013047cd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2158,7 +2158,7 @@
         <x:v>v10.6</x:v>
       </x:c>
       <x:c r="F62" s="54" t="str">
-        <x:v>本机专项4项、类型/格式通过，Lint无错误。相同源码在隔离环境71文件419项、PostgreSQL19项、浏览器16项通过，生产构建及Compose通过。备份5e1ab24e校验67条目通过。生产逐篇验收结果见v10.6发布记录。</x:v>
+        <x:v>相同源码隔离环境419项、PostgreSQL19项、浏览器16项及构建通过。本机类型/格式通过。生产19主题19篇正文HTML不变，元信息/标题入口/目录锚点通过，桌面/手机无溢出。备份67条目校验、数据量不变。代码5ff67ca，详见v10.6发布记录。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix: remove topic heading block and separator (V10.7)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R97058d8e9cd749e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rf54cd8ca65484898"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R683138d4013047cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R3fad87f324794ca9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Re550dbff225d4a45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R4d0efddb4b814740"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2161,6 +2161,26 @@
         <x:v>相同源码隔离环境419项、PostgreSQL19项、浏览器16项及构建通过。本机类型/格式通过。生产19主题19篇正文HTML不变，元信息/标题入口/目录锚点通过，桌面/手机无溢出。备份67条目校验、数据量不变。代码5ff67ca，详见v10.6发布记录。</x:v>
       </x:c>
     </x:row>
+    <x:row r="63" ht="180" customHeight="1">
+      <x:c r="A63" s="53" t="str">
+        <x:v>V10.7</x:v>
+      </x:c>
+      <x:c r="B63" s="52" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C63" s="54" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D63" s="54" t="str">
+        <x:v>按用户截图继续精简主题页，移除知识库路径、可见主题大标题、本主题文章、文章链接索引及下方横线。更新日期、更新人、正文及两侧导航保留。</x:v>
+      </x:c>
+      <x:c r="E63" s="54" t="str">
+        <x:v>v10.7</x:v>
+      </x:c>
+      <x:c r="F63" s="54" t="str">
+        <x:v>本机类型/格式/Lint通过（2项既有警告）。相同源码隔离环境浏览器16项、构建/Compose通过，覆盖标题区移除、目录/分类导航、窄屏与文章保护。备份b16cb3b4校验67条目通过，生产验收结果见v10.7记录。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3157,6 +3177,20 @@
         <x:v>Git标签v10.6定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.6.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="57" ht="70" customHeight="1">
+      <x:c r="A57" s="55" t="str">
+        <x:v>V10.7</x:v>
+      </x:c>
+      <x:c r="B57" s="56" t="str">
+        <x:v>v10.7</x:v>
+      </x:c>
+      <x:c r="C57" s="57" t="str">
+        <x:v>2026-10-29 移除主题正文上方整块标题及横线</x:v>
+      </x:c>
+      <x:c r="D57" s="58" t="str">
+        <x:v>Git标签v10.7定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.7.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record V10.7 header removal acceptance
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R3fad87f324794ca9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Re550dbff225d4a45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R4d0efddb4b814740"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R6f63aa1eb67b49f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R469faadf9cda4927"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rb9cab3a4e00b42e1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2178,7 +2178,7 @@
         <x:v>v10.7</x:v>
       </x:c>
       <x:c r="F63" s="54" t="str">
-        <x:v>本机类型/格式/Lint通过（2项既有警告）。相同源码隔离环境浏览器16项、构建/Compose通过，覆盖标题区移除、目录/分类导航、窄屏与文章保护。备份b16cb3b4校验67条目通过，生产验收结果见v10.7记录。</x:v>
+        <x:v>浏览器16项、构建/类型/格式/Compose通过，Lint无错误。生产19主题19篇无旧标题区/索引/横线，正文HTML不变，首段更新信息、目录锚点保持；桌面/手机实拍无溢出。备份67条目校验、数据量不变。代码4355be8，详见v10.7记录。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: add application center entry (V10.8)
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R6f63aa1eb67b49f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R469faadf9cda4927"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rb9cab3a4e00b42e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R3f080195587f4069"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rcd2da598e2c34ce5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R5c91ebd75dad47a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2181,6 +2181,26 @@
         <x:v>浏览器16项、构建/类型/格式/Compose通过，Lint无错误。生产19主题19篇无旧标题区/索引/横线，正文HTML不变，首段更新信息、目录锚点保持；桌面/手机实拍无溢出。备份67条目校验、数据量不变。代码4355be8，详见v10.7记录。</x:v>
       </x:c>
     </x:row>
+    <x:row r="64" ht="110" customHeight="1">
+      <x:c r="A64" s="53" t="str">
+        <x:v>V10.8</x:v>
+      </x:c>
+      <x:c r="B64" s="52" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C64" s="54" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D64" s="54" t="str">
+        <x:v>顶部导航在模板中心右侧新增应用中心，手机菜单同步；新增需登录的/apps入口页，显示应用陆续上线，后续补充团队Vibe Coding Web应用。</x:v>
+      </x:c>
+      <x:c r="E64" s="54" t="str">
+        <x:v>计划标签v10.8，待部署验收后发布</x:v>
+      </x:c>
+      <x:c r="F64" s="54" t="str">
+        <x:v>本地lint、typecheck、build、导航3项测试及浏览器验收通过；quality-server.local无法解析，部署及GitHub发布待完成。详见docs/operations/releases/v10.8.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3191,6 +3211,20 @@
         <x:v>Git标签v10.7定位完整交付；源码、验收与生产运行记录见docs/operations/releases/v10.7.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="58" ht="70" customHeight="1">
+      <x:c r="A58" s="55" t="str">
+        <x:v>V10.8</x:v>
+      </x:c>
+      <x:c r="B58" s="56" t="str">
+        <x:v>计划v10.8，待部署验收</x:v>
+      </x:c>
+      <x:c r="C58" s="57" t="str">
+        <x:v>新增应用中心导航及入口占位页</x:v>
+      </x:c>
+      <x:c r="D58" s="58" t="str">
+        <x:v>本地提交标题feat: add application center entry (V10.8)；部署及GitHub发布待网络恢复；验收记录见docs/operations/releases/v10.8.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record V10.8 deployment acceptance
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R3f080195587f4069"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rcd2da598e2c34ce5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R5c91ebd75dad47a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R3c6f684b5e6945e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rea40bcceda814a2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R410682acb2984e41"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2195,10 +2195,10 @@
         <x:v>顶部导航在模板中心右侧新增应用中心，手机菜单同步；新增需登录的/apps入口页，显示应用陆续上线，后续补充团队Vibe Coding Web应用。</x:v>
       </x:c>
       <x:c r="E64" s="54" t="str">
-        <x:v>计划标签v10.8，待部署验收后发布</x:v>
+        <x:v>08e8439 / v10.8</x:v>
       </x:c>
       <x:c r="F64" s="54" t="str">
-        <x:v>本地lint、typecheck、build、导航3项测试及浏览器验收通过；quality-server.local无法解析，部署及GitHub发布待完成。详见docs/operations/releases/v10.8.md。</x:v>
+        <x:v>2026-10-30 已备份并部署quality-server，ready200，Web/DB/proxy健康；线上首页最右侧入口、/apps跳转和375px手机菜单验收通过。详见docs/operations/releases/v10.8.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3216,13 +3216,13 @@
         <x:v>V10.8</x:v>
       </x:c>
       <x:c r="B58" s="56" t="str">
-        <x:v>计划v10.8，待部署验收</x:v>
+        <x:v>08e8439 / v10.8</x:v>
       </x:c>
       <x:c r="C58" s="57" t="str">
         <x:v>新增应用中心导航及入口占位页</x:v>
       </x:c>
       <x:c r="D58" s="58" t="str">
-        <x:v>本地提交标题feat: add application center entry (V10.8)；部署及GitHub发布待网络恢复；验收记录见docs/operations/releases/v10.8.md。</x:v>
+        <x:v>2026-10-30 部署验收通过，代码提交08e8439；v10.8定位交付，验收记录见docs/operations/releases/v10.8.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record V10.9 BOF application acceptance
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R3c6f684b5e6945e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Rea40bcceda814a2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R410682acb2984e41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rc1ac12477ee5489f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R181afc98a4854e4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R00b5732547a14876"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -150,7 +150,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="59">
+  <x:cellXfs count="63">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0"/>
@@ -271,6 +271,18 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -2201,6 +2213,26 @@
         <x:v>2026-10-30 已备份并部署quality-server，ready200，Web/DB/proxy健康；线上首页最右侧入口、/apps跳转和375px手机菜单验收通过。详见docs/operations/releases/v10.8.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="59" t="str">
+        <x:v>V10.9</x:v>
+      </x:c>
+      <x:c r="B65" s="60" t="d">
+        <x:v>2026-10-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C65" s="61" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D65" s="61" t="str">
+        <x:v>应用中心首批接入 BOF 箱线图与散点图 V1.1：新增响应式应用卡片、独立说明页、需登录的工具运行页、受保护案例工作簿下载；案例包含完整四张必需工作表，可直接在工具中生成 2 张图。</x:v>
+      </x:c>
+      <x:c r="E65" s="61" t="str">
+        <x:v>f88d572 / v10.9</x:v>
+      </x:c>
+      <x:c r="F65" s="61" t="str">
+        <x:v>本地模块/集成424项、PostgreSQL 19项、BOF专项e2e 3项通过；全量e2e 130通过/3项既有非BOF失败/1跳过；类型、格式、Lint无错误、生产构建及Docker镜像内资产检查通过。未部署生产，详见docs/operations/releases/v10.9.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3225,6 +3257,20 @@
         <x:v>2026-10-30 部署验收通过，代码提交08e8439；v10.8定位交付，验收记录见docs/operations/releases/v10.8.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="59" t="str">
+        <x:v>V10.9</x:v>
+      </x:c>
+      <x:c r="B59" s="61" t="str">
+        <x:v>f88d572 / v10.9</x:v>
+      </x:c>
+      <x:c r="C59" s="60" t="str">
+        <x:v>2026-10-30 BOF 应用集成</x:v>
+      </x:c>
+      <x:c r="D59" s="62" t="str">
+        <x:v>应用中心接入 BOF、受控运行页、使用说明与案例工作簿；Git标签v10.9定位完整交付，验收记录见docs/operations/releases/v10.9.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record V10.9 deployment acceptance
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="Rc1ac12477ee5489f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R181afc98a4854e4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="R00b5732547a14876"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R5bfb40a3201140b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Re3847348f07141ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rf88292736d894ebe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2227,10 +2227,10 @@
         <x:v>应用中心首批接入 BOF 箱线图与散点图 V1.1：新增响应式应用卡片、独立说明页、需登录的工具运行页、受保护案例工作簿下载；案例包含完整四张必需工作表，可直接在工具中生成 2 张图。</x:v>
       </x:c>
       <x:c r="E65" s="61" t="str">
-        <x:v>f88d572 / v10.9</x:v>
+        <x:v>f88d572、e41a6a7 / v10.9</x:v>
       </x:c>
       <x:c r="F65" s="61" t="str">
-        <x:v>本地模块/集成424项、PostgreSQL 19项、BOF专项e2e 3项通过；全量e2e 130通过/3项既有非BOF失败/1跳过；类型、格式、Lint无错误、生产构建及Docker镜像内资产检查通过。未部署生产，详见docs/operations/releases/v10.9.md。</x:v>
+        <x:v>本地模块/集成424项、PostgreSQL 19项、BOF专项e2e 3项通过；类型、格式、Lint无错误、生产构建及Docker资产检查通过。已备份并部署quality-server，V10.8→V10.9，Web/DB/proxy健康、ready200；线上登录页200，应用及运行页未登录均307到相对登录地址，案例下载401且private/no-store。详见docs/operations/releases/v10.9.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3262,13 +3262,13 @@
         <x:v>V10.9</x:v>
       </x:c>
       <x:c r="B59" s="61" t="str">
-        <x:v>f88d572 / v10.9</x:v>
+        <x:v>f88d572、e41a6a7 / v10.9</x:v>
       </x:c>
       <x:c r="C59" s="60" t="str">
         <x:v>2026-10-30 BOF 应用集成</x:v>
       </x:c>
       <x:c r="D59" s="62" t="str">
-        <x:v>应用中心接入 BOF、受控运行页、使用说明与案例工作簿；Git标签v10.9定位完整交付，验收记录见docs/operations/releases/v10.9.md。</x:v>
+        <x:v>应用中心接入 BOF、受控运行页、使用说明与案例工作簿；修复线上未登录跳转内部地址后重新部署，Git标签v10.9定位完整交付，验收记录见docs/operations/releases/v10.9.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record V10.10 deployment acceptance
</commit_message>
<xml_diff>
--- a/Q-Nexus项目变更说明.xlsx
+++ b/Q-Nexus项目变更说明.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R5bfb40a3201140b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="Re3847348f07141ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rf88292736d894ebe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总览" sheetId="1" r:id="R11f6adbf7dd743ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="提交对照" sheetId="2" r:id="R1c6bb41e009b430a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规则" sheetId="3" r:id="Rfa3676d62c7e438d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2233,6 +2233,26 @@
         <x:v>本地模块/集成424项、PostgreSQL 19项、BOF专项e2e 3项通过；类型、格式、Lint无错误、生产构建及Docker资产检查通过。已备份并部署quality-server，V10.8→V10.9，Web/DB/proxy健康、ready200；线上登录页200，应用及运行页未登录均307到相对登录地址，案例下载401且private/no-store。详见docs/operations/releases/v10.9.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="59" t="str">
+        <x:v>V10.10</x:v>
+      </x:c>
+      <x:c r="B66" s="60" t="d">
+        <x:v>2026-10-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C66" s="61" t="str">
+        <x:v>小型修改</x:v>
+      </x:c>
+      <x:c r="D66" s="61" t="str">
+        <x:v>BOF 升级 V1.2：BinPlot 改为可选；不使用分 Bin 时按每个尺寸的 USL/LSL 绘制上下限，不显示 Bin 色带、边界和名称。案例工作簿移除 BinPlot 页签，应用说明同步两种模式。</x:v>
+      </x:c>
+      <x:c r="E66" s="61" t="str">
+        <x:v>b55ed1e / v10.10</x:v>
+      </x:c>
+      <x:c r="F66" s="61" t="str">
+        <x:v>BOF V1.2专项10项、BOF项目全量108项通过；品集本地424项（单线程）、PostgreSQL19项、BOF专项e2e3项、构建/Lint/格式通过。已备份并部署quality-server，V10.9→V10.10，Web/DB/proxy健康、ready200；线上应用/说明/运行页均307登录，案例下载401；镜像内确认BOF V1.2与无BinPlot四页工作簿。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3271,6 +3291,20 @@
         <x:v>应用中心接入 BOF、受控运行页、使用说明与案例工作簿；修复线上未登录跳转内部地址后重新部署，Git标签v10.9定位完整交付，验收记录见docs/operations/releases/v10.9.md。</x:v>
       </x:c>
     </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="59" t="str">
+        <x:v>V10.10</x:v>
+      </x:c>
+      <x:c r="B60" s="61" t="str">
+        <x:v>b55ed1e / v10.10</x:v>
+      </x:c>
+      <x:c r="C60" s="60" t="str">
+        <x:v>2026-10-30 BOF 可选 BinPlot</x:v>
+      </x:c>
+      <x:c r="D60" s="62" t="str">
+        <x:v>BOF V1.2 支持无 BinPlot 的 Spec 上下限模式，品集同步更新应用版本、说明和案例工作簿；已部署并完成线上边界验收，详见 docs/operations/releases/v10.10.md。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>